<commit_message>
OTRC29652E: add new fsx test az-a
</commit_message>
<xml_diff>
--- a/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
+++ b/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C29652e\projects\Assessment\Assessment\Ambiente Productivo\Lift-and-Shift - 18 Servers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6AE92CB-3E34-42FE-94D8-29DCF93D7D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59EE1E2-DD74-45ED-B89F-05E6E68B8379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
     <author>tc={8DA830ED-0AC2-4775-9D26-12BE22978251}</author>
   </authors>
   <commentList>
-    <comment ref="N12" authorId="0" shapeId="0" xr:uid="{8DA830ED-0AC2-4775-9D26-12BE22978251}">
+    <comment ref="M11" authorId="0" shapeId="0" xr:uid="{8DA830ED-0AC2-4775-9D26-12BE22978251}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="97">
   <si>
     <t>This file contains an export of AWS Transform Assessment results for Production Environment (InteliSrcPA).</t>
   </si>
@@ -236,9 +236,6 @@
     <t>Microsoft Windows Server 2022 (64-bit)</t>
   </si>
   <si>
-    <t>PAHWPAPSRC04</t>
-  </si>
-  <si>
     <t>PAHWPAPWFC01</t>
   </si>
   <si>
@@ -314,15 +311,42 @@
     <t>c5a.large</t>
   </si>
   <si>
-    <t>Se despliega como ASG
-APP 1</t>
+    <t>USAEA1PAPWES33</t>
+  </si>
+  <si>
+    <t>USAEA1PAPWES34</t>
+  </si>
+  <si>
+    <t>USAEA1PFSWES08</t>
+  </si>
+  <si>
+    <t>USAEA1PFSWES09</t>
+  </si>
+  <si>
+    <t>USAEA1PWBWES21
+USAEA1PWBWES22</t>
+  </si>
+  <si>
+    <t>USAEA1PWBWES23
+USAEA1PWBWES24</t>
+  </si>
+  <si>
+    <t>USAEA1PWBWES25
+USAEA1PWBWES26</t>
+  </si>
+  <si>
+    <t>USAEA1PWBWES27
+USAEA1PWBWES28</t>
+  </si>
+  <si>
+    <t>USAEA1PWBWES35</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -347,14 +371,8 @@
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -365,12 +383,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -393,18 +405,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -626,7 +639,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="N12" dT="2026-08-17T14:36:17.06" personId="{2A72F2CE-8368-4257-835E-43F3EF0C2274}" id="{8DA830ED-0AC2-4775-9D26-12BE22978251}">
+  <threadedComment ref="M11" dT="2026-08-17T14:36:17.06" personId="{2A72F2CE-8368-4257-835E-43F3EF0C2274}" id="{8DA830ED-0AC2-4775-9D26-12BE22978251}">
     <text>Se remueve por almacenamiento en FSX</text>
   </threadedComment>
 </ThreadedComments>
@@ -2836,1336 +2849,1310 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:W1000"/>
+  <dimension ref="A1:V999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="21" customWidth="1"/>
-    <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="14" width="15" customWidth="1"/>
-    <col min="15" max="15" width="23" customWidth="1"/>
-    <col min="16" max="16" width="26" customWidth="1"/>
-    <col min="17" max="17" width="40" customWidth="1"/>
-    <col min="18" max="18" width="30" customWidth="1"/>
-    <col min="19" max="21" width="40" customWidth="1"/>
-    <col min="22" max="22" width="37" customWidth="1"/>
-    <col min="23" max="23" width="40" customWidth="1"/>
-    <col min="24" max="27" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="23" customWidth="1"/>
+    <col min="15" max="15" width="26" customWidth="1"/>
+    <col min="16" max="16" width="40" customWidth="1"/>
+    <col min="17" max="17" width="30" customWidth="1"/>
+    <col min="18" max="20" width="40" customWidth="1"/>
+    <col min="21" max="21" width="37" customWidth="1"/>
+    <col min="22" max="22" width="40" customWidth="1"/>
+    <col min="23" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>30</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="W1" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="1">
+      <c r="D2" s="4">
         <v>4</v>
       </c>
-      <c r="F2" s="1">
+      <c r="E2" s="4">
         <v>16</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="G2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="H2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="I2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K2" s="1">
+      <c r="J2" s="4">
         <v>2</v>
       </c>
-      <c r="L2" s="1">
+      <c r="K2" s="4">
         <v>16</v>
       </c>
-      <c r="M2" s="1">
+      <c r="L2" s="4">
         <v>520</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="N2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="P2" s="4">
         <v>1332</v>
       </c>
-      <c r="R2" s="1">
+      <c r="Q2" s="4">
         <v>0</v>
       </c>
-      <c r="S2" s="1">
+      <c r="R2" s="4">
         <v>1244</v>
       </c>
-      <c r="T2" s="1">
+      <c r="S2" s="4">
         <v>964</v>
       </c>
-      <c r="U2" s="1">
+      <c r="T2" s="4">
         <v>876</v>
       </c>
-      <c r="V2" s="1">
+      <c r="U2" s="4">
         <v>771</v>
       </c>
-      <c r="W2" s="1">
+      <c r="V2" s="4">
         <v>683</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="1">
+      <c r="D3" s="4">
         <v>4</v>
       </c>
-      <c r="F3" s="1">
+      <c r="E3" s="4">
         <v>16</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="F3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="G3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="H3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="I3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="1">
+      <c r="J3" s="4">
         <v>2</v>
       </c>
-      <c r="L3" s="1">
+      <c r="K3" s="4">
         <v>16</v>
       </c>
-      <c r="M3" s="1">
+      <c r="L3" s="4">
         <v>210</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="N3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="P3" s="4">
         <v>1332</v>
       </c>
-      <c r="R3" s="1">
+      <c r="Q3" s="4">
         <v>0</v>
       </c>
-      <c r="S3" s="1">
+      <c r="R3" s="4">
         <v>1244</v>
       </c>
-      <c r="T3" s="1">
+      <c r="S3" s="4">
         <v>964</v>
       </c>
-      <c r="U3" s="1">
+      <c r="T3" s="4">
         <v>876</v>
       </c>
-      <c r="V3" s="1">
+      <c r="U3" s="4">
         <v>771</v>
       </c>
-      <c r="W3" s="1">
+      <c r="V3" s="4">
         <v>683</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+    <row r="4" spans="1:22" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="B4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="1">
+      <c r="D4" s="4">
         <v>4</v>
       </c>
-      <c r="F4" s="1">
+      <c r="E4" s="4">
         <v>16</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="F4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="G4" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="H4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="I4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="1">
+      <c r="J4" s="4">
         <v>2</v>
       </c>
-      <c r="L4" s="1">
+      <c r="K4" s="4">
         <v>16</v>
       </c>
-      <c r="M4" s="1">
+      <c r="L4" s="4">
         <v>120</v>
       </c>
-      <c r="N4" s="1">
+      <c r="M4" s="4">
         <v>90</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="N4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="P4" s="4">
         <v>1858</v>
       </c>
-      <c r="R4" s="1">
+      <c r="Q4" s="4">
         <v>806</v>
       </c>
-      <c r="S4" s="1">
+      <c r="R4" s="4">
         <v>990</v>
       </c>
-      <c r="T4" s="1">
+      <c r="S4" s="4">
         <v>1490</v>
       </c>
-      <c r="U4" s="1">
+      <c r="T4" s="4">
         <v>622</v>
       </c>
-      <c r="V4" s="1">
+      <c r="U4" s="4">
         <v>1276</v>
       </c>
-      <c r="W4" s="1">
+      <c r="V4" s="4">
         <v>569</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
+    <row r="5" spans="1:22" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B5" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="1">
+      <c r="D5" s="4">
         <v>4</v>
       </c>
-      <c r="F5" s="1">
+      <c r="E5" s="4">
+        <v>8</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="4">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4">
+        <v>8</v>
+      </c>
+      <c r="L5" s="4">
+        <v>80</v>
+      </c>
+      <c r="M5" s="4">
+        <v>95</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>403</v>
+      </c>
+      <c r="R5" s="4">
+        <v>666</v>
+      </c>
+      <c r="S5" s="4">
+        <v>888</v>
+      </c>
+      <c r="T5" s="4">
+        <v>441</v>
+      </c>
+      <c r="U5" s="4">
+        <v>749</v>
+      </c>
+      <c r="V5" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="4">
+        <v>4</v>
+      </c>
+      <c r="E6" s="4">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J6" s="4">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4">
+        <v>8</v>
+      </c>
+      <c r="L6" s="4">
+        <v>80</v>
+      </c>
+      <c r="M6" s="4">
+        <v>300</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>403</v>
+      </c>
+      <c r="R6" s="4">
+        <v>666</v>
+      </c>
+      <c r="S6" s="4">
+        <v>888</v>
+      </c>
+      <c r="T6" s="4">
+        <v>441</v>
+      </c>
+      <c r="U6" s="4">
+        <v>749</v>
+      </c>
+      <c r="V6" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="4">
+        <v>4</v>
+      </c>
+      <c r="E7" s="4">
         <v>16</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="F7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="G7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="H7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="I7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K5" s="1">
+      <c r="J7" s="4">
         <v>2</v>
       </c>
-      <c r="L5" s="1">
+      <c r="K7" s="4">
         <v>16</v>
       </c>
-      <c r="M5" s="1">
+      <c r="L7" s="4">
         <v>120</v>
       </c>
-      <c r="N5" s="1">
+      <c r="M7" s="4">
         <v>90</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="N7" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="P7" s="4">
         <v>1858</v>
       </c>
-      <c r="R5" s="1">
+      <c r="Q7" s="4">
         <v>806</v>
       </c>
-      <c r="S5" s="1">
+      <c r="R7" s="4">
         <v>990</v>
       </c>
-      <c r="T5" s="1">
+      <c r="S7" s="4">
         <v>1490</v>
       </c>
-      <c r="U5" s="1">
+      <c r="T7" s="4">
         <v>622</v>
       </c>
-      <c r="V5" s="1">
+      <c r="U7" s="4">
         <v>1276</v>
       </c>
-      <c r="W5" s="1">
+      <c r="V7" s="4">
         <v>569</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
+    <row r="8" spans="1:22" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="4">
+        <v>4</v>
+      </c>
+      <c r="E8" s="4">
+        <v>8</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" s="4">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4">
+        <v>8</v>
+      </c>
+      <c r="L8" s="4">
+        <v>120</v>
+      </c>
+      <c r="M8" s="4">
+        <v>90</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P8" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>403</v>
+      </c>
+      <c r="R8" s="4">
+        <v>666</v>
+      </c>
+      <c r="S8" s="4">
+        <v>888</v>
+      </c>
+      <c r="T8" s="4">
+        <v>441</v>
+      </c>
+      <c r="U8" s="4">
+        <v>749</v>
+      </c>
+      <c r="V8" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="4">
+        <v>4</v>
+      </c>
+      <c r="E9" s="4">
+        <v>8</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="4">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4">
+        <v>8</v>
+      </c>
+      <c r="L9" s="4">
+        <v>120</v>
+      </c>
+      <c r="M9" s="4">
+        <v>90</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q9" s="4">
+        <v>403</v>
+      </c>
+      <c r="R9" s="4">
+        <v>666</v>
+      </c>
+      <c r="S9" s="4">
+        <v>888</v>
+      </c>
+      <c r="T9" s="4">
+        <v>441</v>
+      </c>
+      <c r="U9" s="4">
+        <v>749</v>
+      </c>
+      <c r="V9" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="4">
+        <v>4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>16</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" s="4">
+        <v>2</v>
+      </c>
+      <c r="K10" s="4">
+        <v>16</v>
+      </c>
+      <c r="L10" s="4">
+        <v>120</v>
+      </c>
+      <c r="M10" s="4">
+        <v>90</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P10" s="4">
+        <v>1858</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>806</v>
+      </c>
+      <c r="R10" s="4">
+        <v>990</v>
+      </c>
+      <c r="S10" s="4">
+        <v>1490</v>
+      </c>
+      <c r="T10" s="4">
+        <v>622</v>
+      </c>
+      <c r="U10" s="4">
+        <v>1276</v>
+      </c>
+      <c r="V10" s="4">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="4">
+        <v>4</v>
+      </c>
+      <c r="E11" s="4">
+        <v>8</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" s="4">
+        <v>1</v>
+      </c>
+      <c r="K11" s="4">
+        <v>8</v>
+      </c>
+      <c r="L11" s="4">
+        <v>120</v>
+      </c>
+      <c r="M11" s="4">
+        <v>90</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P11" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>403</v>
+      </c>
+      <c r="R11" s="4">
+        <v>666</v>
+      </c>
+      <c r="S11" s="4">
+        <v>888</v>
+      </c>
+      <c r="T11" s="4">
+        <v>441</v>
+      </c>
+      <c r="U11" s="4">
+        <v>749</v>
+      </c>
+      <c r="V11" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="4">
+        <v>4</v>
+      </c>
+      <c r="E12" s="4">
+        <v>8</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" s="4">
+        <v>1</v>
+      </c>
+      <c r="K12" s="4">
+        <v>8</v>
+      </c>
+      <c r="L12" s="4">
+        <v>120</v>
+      </c>
+      <c r="M12" s="4">
+        <v>90</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P12" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>403</v>
+      </c>
+      <c r="R12" s="4">
+        <v>666</v>
+      </c>
+      <c r="S12" s="4">
+        <v>888</v>
+      </c>
+      <c r="T12" s="4">
+        <v>441</v>
+      </c>
+      <c r="U12" s="4">
+        <v>749</v>
+      </c>
+      <c r="V12" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="4">
+        <v>4</v>
+      </c>
+      <c r="E13" s="4">
+        <v>8</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4">
+        <v>8</v>
+      </c>
+      <c r="L13" s="4">
+        <v>120</v>
+      </c>
+      <c r="M13" s="4">
+        <v>90</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P13" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q13" s="4">
+        <v>403</v>
+      </c>
+      <c r="R13" s="4">
+        <v>666</v>
+      </c>
+      <c r="S13" s="4">
+        <v>888</v>
+      </c>
+      <c r="T13" s="4">
+        <v>441</v>
+      </c>
+      <c r="U13" s="4">
+        <v>749</v>
+      </c>
+      <c r="V13" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="4">
+        <v>4</v>
+      </c>
+      <c r="E14" s="4">
+        <v>8</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="H14" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J14" s="4">
+        <v>1</v>
+      </c>
+      <c r="K14" s="4">
+        <v>8</v>
+      </c>
+      <c r="L14" s="4">
+        <v>80</v>
+      </c>
+      <c r="M14" s="4">
+        <v>90</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P14" s="4">
+        <v>1113</v>
+      </c>
+      <c r="Q14" s="4">
+        <v>403</v>
+      </c>
+      <c r="R14" s="4">
+        <v>666</v>
+      </c>
+      <c r="S14" s="4">
+        <v>888</v>
+      </c>
+      <c r="T14" s="4">
+        <v>441</v>
+      </c>
+      <c r="U14" s="4">
+        <v>749</v>
+      </c>
+      <c r="V14" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E6" s="1">
+      <c r="D15" s="4">
+        <v>2</v>
+      </c>
+      <c r="E15" s="4">
+        <v>8</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="4">
+        <v>2</v>
+      </c>
+      <c r="K15" s="4">
+        <v>8</v>
+      </c>
+      <c r="L15" s="4">
+        <v>90</v>
+      </c>
+      <c r="M15" s="4">
+        <v>150</v>
+      </c>
+      <c r="N15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P15" s="4">
+        <v>942</v>
+      </c>
+      <c r="Q15" s="4">
+        <v>242</v>
+      </c>
+      <c r="R15" s="4">
+        <v>659</v>
+      </c>
+      <c r="S15" s="4">
+        <v>696</v>
+      </c>
+      <c r="T15" s="4">
+        <v>413</v>
+      </c>
+      <c r="U15" s="4">
+        <v>568</v>
+      </c>
+      <c r="V15" s="4">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="4">
         <v>4</v>
       </c>
-      <c r="F6" s="1">
+      <c r="E16" s="4">
+        <v>16</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J16" s="4">
+        <v>2</v>
+      </c>
+      <c r="K16" s="4">
+        <v>16</v>
+      </c>
+      <c r="L16" s="4">
+        <v>120</v>
+      </c>
+      <c r="M16" s="4">
+        <v>180</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P16" s="4">
+        <v>1858</v>
+      </c>
+      <c r="Q16" s="4">
+        <v>806</v>
+      </c>
+      <c r="R16" s="4">
+        <v>990</v>
+      </c>
+      <c r="S16" s="4">
+        <v>1490</v>
+      </c>
+      <c r="T16" s="4">
+        <v>622</v>
+      </c>
+      <c r="U16" s="4">
+        <v>1276</v>
+      </c>
+      <c r="V16" s="4">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="4">
+        <v>4</v>
+      </c>
+      <c r="E17" s="4">
+        <v>16</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J17" s="4">
+        <v>2</v>
+      </c>
+      <c r="K17" s="4">
+        <v>16</v>
+      </c>
+      <c r="L17" s="4">
+        <v>120</v>
+      </c>
+      <c r="M17" s="4">
+        <v>90</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P17" s="4">
+        <v>1858</v>
+      </c>
+      <c r="Q17" s="4">
+        <v>806</v>
+      </c>
+      <c r="R17" s="4">
+        <v>990</v>
+      </c>
+      <c r="S17" s="4">
+        <v>1490</v>
+      </c>
+      <c r="T17" s="4">
+        <v>622</v>
+      </c>
+      <c r="U17" s="4">
+        <v>1276</v>
+      </c>
+      <c r="V17" s="4">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="4">
+        <v>4</v>
+      </c>
+      <c r="E18" s="4">
+        <v>16</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18" s="4">
+        <v>2</v>
+      </c>
+      <c r="K18" s="4">
+        <v>16</v>
+      </c>
+      <c r="L18" s="4">
+        <v>120</v>
+      </c>
+      <c r="M18" s="4">
+        <v>90</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P18" s="4">
+        <v>1858</v>
+      </c>
+      <c r="Q18" s="4">
+        <v>806</v>
+      </c>
+      <c r="R18" s="4">
+        <v>990</v>
+      </c>
+      <c r="S18" s="4">
+        <v>1490</v>
+      </c>
+      <c r="T18" s="4">
+        <v>622</v>
+      </c>
+      <c r="U18" s="4">
+        <v>1276</v>
+      </c>
+      <c r="V18" s="4">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="4">
+        <v>4</v>
+      </c>
+      <c r="E19" s="4">
         <v>8</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="F19" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="G19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1</v>
-      </c>
-      <c r="L6" s="1">
+      <c r="I19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J19" s="4">
+        <v>4</v>
+      </c>
+      <c r="K19" s="4">
         <v>8</v>
       </c>
-      <c r="M6" s="1">
-        <v>80</v>
-      </c>
-      <c r="N6" s="1">
-        <v>95</v>
-      </c>
-      <c r="O6" s="1" t="s">
+      <c r="L19" s="4">
+        <v>280</v>
+      </c>
+      <c r="N19" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q6" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R6" s="1">
-        <v>403</v>
-      </c>
-      <c r="S6" s="1">
-        <v>666</v>
-      </c>
-      <c r="T6" s="1">
-        <v>888</v>
-      </c>
-      <c r="U6" s="1">
-        <v>441</v>
-      </c>
-      <c r="V6" s="1">
-        <v>749</v>
-      </c>
-      <c r="W6" s="1">
-        <v>302</v>
-      </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="1" t="s">
+    <row r="20" spans="1:22" s="3" customFormat="1" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="1">
+      <c r="D20" s="4">
         <v>4</v>
       </c>
-      <c r="F7" s="1">
+      <c r="E20" s="4">
         <v>8</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="F20" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="G20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K7" s="1">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1">
+      <c r="I20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J20" s="4">
+        <v>4</v>
+      </c>
+      <c r="K20" s="4">
         <v>8</v>
       </c>
-      <c r="M7" s="1">
-        <v>80</v>
-      </c>
-      <c r="N7" s="1">
-        <v>300</v>
-      </c>
-      <c r="O7" s="1" t="s">
+      <c r="L20" s="4">
+        <v>200</v>
+      </c>
+      <c r="N20" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q7" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R7" s="1">
-        <v>403</v>
-      </c>
-      <c r="S7" s="1">
-        <v>666</v>
-      </c>
-      <c r="T7" s="1">
-        <v>888</v>
-      </c>
-      <c r="U7" s="1">
-        <v>441</v>
-      </c>
-      <c r="V7" s="1">
-        <v>749</v>
-      </c>
-      <c r="W7" s="1">
-        <v>302</v>
-      </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="1" t="s">
+    <row r="21" spans="1:22" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="1">
+      <c r="D21" s="4">
         <v>4</v>
       </c>
-      <c r="F8" s="1">
-        <v>16</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" s="1">
+      <c r="E21" s="4">
         <v>2</v>
       </c>
-      <c r="L8" s="1">
-        <v>16</v>
-      </c>
-      <c r="M8" s="1">
-        <v>120</v>
-      </c>
-      <c r="N8" s="1">
-        <v>90</v>
-      </c>
-      <c r="O8" s="1" t="s">
+      <c r="F21" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J21" s="4">
+        <v>2</v>
+      </c>
+      <c r="K21" s="4">
+        <v>4</v>
+      </c>
+      <c r="L21" s="4">
+        <v>210</v>
+      </c>
+      <c r="N21" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Q8" s="1">
-        <v>1858</v>
-      </c>
-      <c r="R8" s="1">
-        <v>806</v>
-      </c>
-      <c r="S8" s="1">
-        <v>990</v>
-      </c>
-      <c r="T8" s="1">
-        <v>1490</v>
-      </c>
-      <c r="U8" s="1">
-        <v>622</v>
-      </c>
-      <c r="V8" s="1">
-        <v>1276</v>
-      </c>
-      <c r="W8" s="1">
-        <v>569</v>
-      </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" s="1">
-        <v>4</v>
-      </c>
-      <c r="F9" s="1">
-        <v>8</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K9" s="1">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1">
-        <v>8</v>
-      </c>
-      <c r="M9" s="1">
-        <v>120</v>
-      </c>
-      <c r="N9" s="1">
-        <v>90</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q9" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R9" s="1">
-        <v>403</v>
-      </c>
-      <c r="S9" s="1">
-        <v>666</v>
-      </c>
-      <c r="T9" s="1">
-        <v>888</v>
-      </c>
-      <c r="U9" s="1">
-        <v>441</v>
-      </c>
-      <c r="V9" s="1">
-        <v>749</v>
-      </c>
-      <c r="W9" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="1">
-        <v>4</v>
-      </c>
-      <c r="F10" s="1">
-        <v>8</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K10" s="1">
-        <v>1</v>
-      </c>
-      <c r="L10" s="1">
-        <v>8</v>
-      </c>
-      <c r="M10" s="1">
-        <v>120</v>
-      </c>
-      <c r="N10" s="1">
-        <v>90</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R10" s="1">
-        <v>403</v>
-      </c>
-      <c r="S10" s="1">
-        <v>666</v>
-      </c>
-      <c r="T10" s="1">
-        <v>888</v>
-      </c>
-      <c r="U10" s="1">
-        <v>441</v>
-      </c>
-      <c r="V10" s="1">
-        <v>749</v>
-      </c>
-      <c r="W10" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="1">
-        <v>4</v>
-      </c>
-      <c r="F11" s="1">
-        <v>16</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K11" s="1">
-        <v>2</v>
-      </c>
-      <c r="L11" s="1">
-        <v>16</v>
-      </c>
-      <c r="M11" s="1">
-        <v>120</v>
-      </c>
-      <c r="N11" s="1">
-        <v>90</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>1858</v>
-      </c>
-      <c r="R11" s="1">
-        <v>806</v>
-      </c>
-      <c r="S11" s="1">
-        <v>990</v>
-      </c>
-      <c r="T11" s="1">
-        <v>1490</v>
-      </c>
-      <c r="U11" s="1">
-        <v>622</v>
-      </c>
-      <c r="V11" s="1">
-        <v>1276</v>
-      </c>
-      <c r="W11" s="1">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="4">
-        <v>4</v>
-      </c>
-      <c r="F12" s="4">
-        <v>8</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="K12" s="4">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4">
-        <v>8</v>
-      </c>
-      <c r="M12" s="4">
-        <v>120</v>
-      </c>
-      <c r="N12" s="4">
-        <v>90</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q12" s="4">
-        <v>1113</v>
-      </c>
-      <c r="R12" s="4">
-        <v>403</v>
-      </c>
-      <c r="S12" s="4">
-        <v>666</v>
-      </c>
-      <c r="T12" s="4">
-        <v>888</v>
-      </c>
-      <c r="U12" s="4">
-        <v>441</v>
-      </c>
-      <c r="V12" s="4">
-        <v>749</v>
-      </c>
-      <c r="W12" s="4">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="1">
-        <v>4</v>
-      </c>
-      <c r="F13" s="1">
-        <v>8</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K13" s="1">
-        <v>1</v>
-      </c>
-      <c r="L13" s="1">
-        <v>8</v>
-      </c>
-      <c r="M13" s="1">
-        <v>120</v>
-      </c>
-      <c r="N13" s="1">
-        <v>90</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R13" s="1">
-        <v>403</v>
-      </c>
-      <c r="S13" s="1">
-        <v>666</v>
-      </c>
-      <c r="T13" s="1">
-        <v>888</v>
-      </c>
-      <c r="U13" s="1">
-        <v>441</v>
-      </c>
-      <c r="V13" s="1">
-        <v>749</v>
-      </c>
-      <c r="W13" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="1">
-        <v>4</v>
-      </c>
-      <c r="F14" s="1">
-        <v>8</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1</v>
-      </c>
-      <c r="L14" s="1">
-        <v>8</v>
-      </c>
-      <c r="M14" s="1">
-        <v>120</v>
-      </c>
-      <c r="N14" s="1">
-        <v>90</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q14" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R14" s="1">
-        <v>403</v>
-      </c>
-      <c r="S14" s="1">
-        <v>666</v>
-      </c>
-      <c r="T14" s="1">
-        <v>888</v>
-      </c>
-      <c r="U14" s="1">
-        <v>441</v>
-      </c>
-      <c r="V14" s="1">
-        <v>749</v>
-      </c>
-      <c r="W14" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E15" s="1">
-        <v>4</v>
-      </c>
-      <c r="F15" s="1">
-        <v>8</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K15" s="1">
-        <v>1</v>
-      </c>
-      <c r="L15" s="1">
-        <v>8</v>
-      </c>
-      <c r="M15" s="1">
-        <v>80</v>
-      </c>
-      <c r="N15" s="1">
-        <v>90</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q15" s="1">
-        <v>1113</v>
-      </c>
-      <c r="R15" s="1">
-        <v>403</v>
-      </c>
-      <c r="S15" s="1">
-        <v>666</v>
-      </c>
-      <c r="T15" s="1">
-        <v>888</v>
-      </c>
-      <c r="U15" s="1">
-        <v>441</v>
-      </c>
-      <c r="V15" s="1">
-        <v>749</v>
-      </c>
-      <c r="W15" s="1">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="1">
-        <v>2</v>
-      </c>
-      <c r="F16" s="1">
-        <v>8</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="K16" s="1">
-        <v>2</v>
-      </c>
-      <c r="L16" s="1">
-        <v>8</v>
-      </c>
-      <c r="M16" s="1">
-        <v>90</v>
-      </c>
-      <c r="N16" s="1">
-        <v>150</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>942</v>
-      </c>
-      <c r="R16" s="1">
-        <v>242</v>
-      </c>
-      <c r="S16" s="1">
-        <v>659</v>
-      </c>
-      <c r="T16" s="1">
-        <v>696</v>
-      </c>
-      <c r="U16" s="1">
-        <v>413</v>
-      </c>
-      <c r="V16" s="1">
-        <v>568</v>
-      </c>
-      <c r="W16" s="1">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="1">
-        <v>4</v>
-      </c>
-      <c r="F17" s="1">
-        <v>16</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K17" s="1">
-        <v>2</v>
-      </c>
-      <c r="L17" s="1">
-        <v>16</v>
-      </c>
-      <c r="M17" s="1">
-        <v>120</v>
-      </c>
-      <c r="N17" s="1">
-        <v>180</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>1858</v>
-      </c>
-      <c r="R17" s="1">
-        <v>806</v>
-      </c>
-      <c r="S17" s="1">
-        <v>990</v>
-      </c>
-      <c r="T17" s="1">
-        <v>1490</v>
-      </c>
-      <c r="U17" s="1">
-        <v>622</v>
-      </c>
-      <c r="V17" s="1">
-        <v>1276</v>
-      </c>
-      <c r="W17" s="1">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="1">
-        <v>4</v>
-      </c>
-      <c r="F18" s="1">
-        <v>16</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K18" s="1">
-        <v>2</v>
-      </c>
-      <c r="L18" s="1">
-        <v>16</v>
-      </c>
-      <c r="M18" s="1">
-        <v>120</v>
-      </c>
-      <c r="N18" s="1">
-        <v>90</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>1858</v>
-      </c>
-      <c r="R18" s="1">
-        <v>806</v>
-      </c>
-      <c r="S18" s="1">
-        <v>990</v>
-      </c>
-      <c r="T18" s="1">
-        <v>1490</v>
-      </c>
-      <c r="U18" s="1">
-        <v>622</v>
-      </c>
-      <c r="V18" s="1">
-        <v>1276</v>
-      </c>
-      <c r="W18" s="1">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="1">
-        <v>4</v>
-      </c>
-      <c r="F19" s="1">
-        <v>16</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K19" s="1">
-        <v>2</v>
-      </c>
-      <c r="L19" s="1">
-        <v>16</v>
-      </c>
-      <c r="M19" s="1">
-        <v>120</v>
-      </c>
-      <c r="N19" s="1">
-        <v>90</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>1858</v>
-      </c>
-      <c r="R19" s="1">
-        <v>806</v>
-      </c>
-      <c r="S19" s="1">
-        <v>990</v>
-      </c>
-      <c r="T19" s="1">
-        <v>1490</v>
-      </c>
-      <c r="U19" s="1">
-        <v>622</v>
-      </c>
-      <c r="V19" s="1">
-        <v>1276</v>
-      </c>
-      <c r="W19" s="1">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="1">
-        <v>4</v>
-      </c>
-      <c r="F20" s="1">
-        <v>8</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K20" s="1">
-        <v>4</v>
-      </c>
-      <c r="L20" s="1">
-        <v>8</v>
-      </c>
-      <c r="M20" s="1">
-        <v>280</v>
-      </c>
-      <c r="O20" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E21" s="1">
-        <v>4</v>
-      </c>
-      <c r="F21" s="1">
-        <v>8</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="K21" s="1">
-        <v>4</v>
-      </c>
-      <c r="L21" s="1">
-        <v>8</v>
-      </c>
-      <c r="M21" s="1">
-        <v>200</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E22" s="1">
-        <v>4</v>
-      </c>
-      <c r="F22" s="1">
-        <v>2</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K22" s="1">
-        <v>2</v>
-      </c>
-      <c r="L22" s="1">
-        <v>4</v>
-      </c>
-      <c r="M22" s="1">
-        <v>210</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5133,7 +5120,6 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
feat: update tco prod
</commit_message>
<xml_diff>
--- a/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
+++ b/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
@@ -1,407 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C29652e\projects\Assessment\Assessment\Ambiente Productivo\Lift-and-Shift - 18 Servers\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A89306-F27B-4B64-A87D-EBDEE10D4C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" r:id="rId1"/>
-    <sheet name="Glossary" sheetId="2" r:id="rId2"/>
-    <sheet name="Shared Tenancy Analysis" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Tenancy Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="114">
-  <si>
-    <t>Host Name Onpremise</t>
-  </si>
-  <si>
-    <t>EC2 Name</t>
-  </si>
-  <si>
-    <t>Enviroment</t>
-  </si>
-  <si>
-    <t>Number of CPUs</t>
-  </si>
-  <si>
-    <t>RAM (GB)</t>
-  </si>
-  <si>
-    <t>Operation System Type</t>
-  </si>
-  <si>
-    <t>Operation System Name</t>
-  </si>
-  <si>
-    <t>AWS Instance Recommended</t>
-  </si>
-  <si>
-    <t>AWS Instance Deploy</t>
-  </si>
-  <si>
-    <t>AWS Total Cores</t>
-  </si>
-  <si>
-    <t>AWS RAM (GB)</t>
-  </si>
-  <si>
-    <t>EBS Size (GB)</t>
-  </si>
-  <si>
-    <t>AWS Region</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr EBS Cost</t>
-  </si>
-  <si>
-    <t>Annualized On-Demand Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized License Only Cost</t>
-  </si>
-  <si>
-    <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
-  </si>
-  <si>
-    <t>Annualized 3 Yr NURI Total EC2 Cost</t>
-  </si>
-  <si>
-    <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
-  </si>
-  <si>
-    <t>PAHWPAPSTS01</t>
-  </si>
-  <si>
-    <t>PROD</t>
-  </si>
-  <si>
-    <t>RHEL</t>
-  </si>
-  <si>
-    <t>Red Hat Enterprise Linux 8 (64-bit)</t>
-  </si>
-  <si>
-    <t>r5a.large</t>
-  </si>
-  <si>
-    <t>US East (N. Virginia)</t>
-  </si>
-  <si>
-    <t>PAHWPAPSTE01</t>
-  </si>
-  <si>
-    <t>PAHWPAPSRC03</t>
-  </si>
-  <si>
-    <t>Windows</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2022 (64-bit)</t>
-  </si>
-  <si>
-    <t>PAHWPAPWFC01</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2019 (64-bit)</t>
-  </si>
-  <si>
-    <t>r7a.medium</t>
-  </si>
-  <si>
-    <t>PAHWPWFINT01</t>
-  </si>
-  <si>
-    <t>USAEA1PFSWES09</t>
-  </si>
-  <si>
-    <t>PAHWPWSAPI01</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES35</t>
-  </si>
-  <si>
-    <t>PAHWPAPWSS03</t>
-  </si>
-  <si>
-    <t>PAHWPAPWEF02</t>
-  </si>
-  <si>
-    <t>USAEA1PAPWES34</t>
-  </si>
-  <si>
-    <t>PAHWPAPTUI03</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2022 (64-bit) [ASG app1 desplegado]</t>
-  </si>
-  <si>
-    <t>PAHWPCHECS01</t>
-  </si>
-  <si>
-    <t>USAEA1PFSWES08</t>
-  </si>
-  <si>
-    <t>pahqpapapp02</t>
-  </si>
-  <si>
-    <t>USAEA1PAPWES33</t>
-  </si>
-  <si>
-    <t>Windows Server 2019 Standard</t>
-  </si>
-  <si>
-    <t>pahwpapbof01</t>
-  </si>
-  <si>
-    <t>Linux</t>
-  </si>
-  <si>
-    <t>Ubuntu 22.04.3 LTS</t>
-  </si>
-  <si>
-    <t>c5a.large</t>
-  </si>
-  <si>
-    <t>RDS produccion (multiaz1)</t>
-  </si>
-  <si>
-    <t>SQL Server - Standard</t>
-  </si>
-  <si>
-    <t>SQL Server Standard Edition 15.x (Multi-AZ, license-included)</t>
-  </si>
-  <si>
-    <t>db.r6i.4xlarge</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>RDS procesos (standalone1)</t>
-  </si>
-  <si>
-    <t>SQL Server Standard Edition 15.x (Single-AZ, license-included)</t>
-  </si>
-  <si>
-    <t>db.r6i.2xlarge</t>
-  </si>
-  <si>
-    <t>FSx Windows (intelisrcpa-prd)</t>
-  </si>
-  <si>
-    <t>Windows (FSx)</t>
-  </si>
-  <si>
-    <t>FSx Windows File Server Single-AZ SSD (64 MBps, backup 30d)</t>
-  </si>
-  <si>
-    <t>FSx SINGLE_AZ_1</t>
-  </si>
-  <si>
-    <t>AMI Builder (temporal)</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2025 (AMI Builder - temporal)</t>
-  </si>
-  <si>
-    <t>m5.large</t>
-  </si>
-  <si>
-    <t>DMS replication (poc)</t>
-  </si>
-  <si>
-    <t>DMS</t>
-  </si>
-  <si>
-    <t>DMS c5.2xlarge Single-AZ (engine 3.6.1)</t>
-  </si>
-  <si>
-    <t>dms.c5.2xlarge</t>
-  </si>
-  <si>
-    <t>This file contains an export of AWS Transform Assessment results for Production Environment (InteliSrcPA).</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Glossary</t>
-  </si>
-  <si>
-    <t>Column-by-column definitions and descriptions for all data fields.</t>
-  </si>
-  <si>
-    <t>Shared Tenancy Analysis</t>
-  </si>
-  <si>
-    <t>Lists servers that can run on shared hardware infrastructure in AWS.</t>
-  </si>
-  <si>
-    <t>Attribute Name</t>
-  </si>
-  <si>
-    <t>Name assigned to the server on-premise</t>
-  </si>
-  <si>
-    <t>Name for the EC2 instance in AWS</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Production/Development/Test environment designation</t>
-  </si>
-  <si>
-    <t>Count of virtual processors</t>
-  </si>
-  <si>
-    <t>Total memory capacity in gigabytes</t>
-  </si>
-  <si>
-    <t>Category of operating system</t>
-  </si>
-  <si>
-    <t>Specific OS version/distribution</t>
-  </si>
-  <si>
-    <t>Recommended AWS instance type by assessment tool</t>
-  </si>
-  <si>
-    <t>Instance type to be deployed</t>
-  </si>
-  <si>
-    <t>Total cores in recommended EC2 instance</t>
-  </si>
-  <si>
-    <t>Memory in recommended instance in GB</t>
-  </si>
-  <si>
-    <t>Root volume EBS storage size in GB</t>
-  </si>
-  <si>
-    <t>EBS Size (GB) Additional</t>
-  </si>
-  <si>
-    <t>Additional EBS volumes in GB</t>
-  </si>
-  <si>
-    <t>Target AWS geographic region</t>
-  </si>
-  <si>
-    <t>Yearly EBS storage cost</t>
-  </si>
-  <si>
-    <t>Yearly total cost using on-demand pricing</t>
-  </si>
-  <si>
-    <t>Yearly licensing costs</t>
-  </si>
-  <si>
-    <t>Yearly compute costs at on-demand rates</t>
-  </si>
-  <si>
-    <t>Total yearly cost with 1-year RI no upfront</t>
-  </si>
-  <si>
-    <t>Compute-only yearly cost with 1-year RI</t>
-  </si>
-  <si>
-    <t>Total yearly cost with 3-year RI no upfront</t>
-  </si>
-  <si>
-    <t>Compute-only yearly cost with 3-year RI</t>
-  </si>
-  <si>
-    <t>EBS Additional Size (GB)</t>
-  </si>
-  <si>
-    <t>Monthly Root EBS Cost</t>
-  </si>
-  <si>
-    <t>Monthly Additional EBS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr Additional EBS Cost</t>
-  </si>
-  <si>
-    <t>Monthly  On-Demand Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Monthly 1 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Monthly 3 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES23 
-USAEA1PWBWES24</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES25 
-USAEA1PWBWES26</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES27 
-USAEA1PWBWES28</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES21 
-USAEA1PWBWES22</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Amazon Ember"/>
+      <b val="1"/>
+      <color theme="0"/>
       <sz val="12"/>
-      <color theme="0"/>
-      <name val="Amazon Ember"/>
     </font>
     <font>
+      <name val="Amazon Ember"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Amazon Ember"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -457,40 +101,99 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -691,40 +394,58 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="8.7109375" customWidth="1"/>
+    <col width="8.7109375" customWidth="1" min="1" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>71</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>This file contains an export of AWS Transform Assessment results for Production Environment (InteliSrcPA).</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>73</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>75</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Glossary</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Column-by-column definitions and descriptions for all data fields.</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>77</v>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Shared Tenancy Analysis</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Lists servers that can run on shared hardware infrastructure in AWS.</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1714,210 +1435,308 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="8.7109375" customWidth="1"/>
+    <col width="8.7109375" customWidth="1" min="1" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>73</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Attribute Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>76</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Shared Tenancy Analysis</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>79</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Host Name Onpremise</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Name assigned to the server on-premise</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>80</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EC2 Name</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Name for the EC2 instance in AWS</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>82</v>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Production/Development/Test environment designation</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>83</v>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Number of CPUs</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Count of virtual processors</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>84</v>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>RAM (GB)</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Total memory capacity in gigabytes</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>85</v>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Operation System Type</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Category of operating system</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>86</v>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Operation System Name</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Specific OS version/distribution</t>
+        </is>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>87</v>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>AWS Instance Recommended</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Recommended AWS instance type by assessment tool</t>
+        </is>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>88</v>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>AWS Instance Deploy</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Instance type to be deployed</t>
+        </is>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>89</v>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>AWS Total Cores</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Total cores in recommended EC2 instance</t>
+        </is>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>90</v>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>AWS RAM (GB)</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Memory in recommended instance in GB</t>
+        </is>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>91</v>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>EBS Size (GB)</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Root volume EBS storage size in GB</t>
+        </is>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>93</v>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>EBS Size (GB) Additional</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Additional EBS volumes in GB</t>
+        </is>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>94</v>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>AWS Region</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Target AWS geographic region</t>
+        </is>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>95</v>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr EBS Cost</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Yearly EBS storage cost</t>
+        </is>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>96</v>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Yearly total cost using on-demand pricing</t>
+        </is>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>97</v>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Annualized License Only Cost</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Yearly licensing costs</t>
+        </is>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>98</v>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Yearly compute costs at on-demand rates</t>
+        </is>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>99</v>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Total yearly cost with 1-year RI no upfront</t>
+        </is>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A22" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>100</v>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Compute-only yearly cost with 1-year RI</t>
+        </is>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>101</v>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI Total EC2 Cost</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Total yearly cost with 3-year RI no upfront</t>
+        </is>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A24" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>102</v>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Compute-only yearly cost with 3-year RI</t>
+        </is>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:2" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2893,1329 +2712,1804 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AB999"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="67.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23" customWidth="1"/>
-    <col min="15" max="15" width="27.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26" customWidth="1"/>
-    <col min="17" max="17" width="33.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="48.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="40" customWidth="1"/>
-    <col min="21" max="21" width="30" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="40" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="79.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="40" customWidth="1"/>
-    <col min="25" max="25" width="40" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="79.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="37" customWidth="1"/>
-    <col min="28" max="28" width="40" hidden="1" customWidth="1"/>
-    <col min="29" max="32" width="8.7109375" customWidth="1"/>
+    <col width="31.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="48.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="27.140625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="67.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="34.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="25" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="19.85546875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="17.85546875" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="17" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="28.85546875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="27.42578125" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="33.28515625" bestFit="1" customWidth="1" style="6" min="17" max="17"/>
+    <col width="41.7109375" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="48.85546875" bestFit="1" customWidth="1" style="6" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="30" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="40" customWidth="1" min="22" max="22"/>
+    <col width="79.85546875" bestFit="1" customWidth="1" style="6" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col hidden="1" width="40" customWidth="1" min="25" max="25"/>
+    <col width="79.85546875" bestFit="1" customWidth="1" style="6" min="26" max="26"/>
+    <col width="37" customWidth="1" min="27" max="27"/>
+    <col hidden="1" width="40" customWidth="1" min="28" max="28"/>
+    <col width="8.7109375" customWidth="1" min="29" max="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="15.75" customFormat="1" customHeight="1" s="6">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Host Name Onpremise</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>EC2 Name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Enviroment</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Number of CPUs</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>RAM (GB)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Operation System Type</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Operation System Name</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Instance Recommended</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>AWS Instance Deploy</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Total Cores</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>AWS RAM (GB)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>EBS Size (GB)</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>EBS Additional Size (GB)</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Region</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly Root EBS Cost</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr EBS Cost</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly Additional EBS Cost</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr Additional EBS Cost</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly  On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized License Only Cost</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly 1 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly 3 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI Total EC2 Cost</t>
+        </is>
+      </c>
+      <c r="AB1" s="6" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPAPSTS01</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>RHEL</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 8 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>520</v>
+      </c>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P2" s="7" t="n">
+        <v>499.2</v>
+      </c>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n">
+        <v>111</v>
+      </c>
+      <c r="T2" s="7" t="n">
+        <v>1332</v>
+      </c>
+      <c r="U2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="V2" s="7" t="n">
+        <v>1244</v>
+      </c>
+      <c r="W2" s="7" t="n">
+        <v>80.33</v>
+      </c>
+      <c r="X2" s="7" t="n">
+        <v>964</v>
+      </c>
+      <c r="Y2" s="7" t="n">
+        <v>876</v>
+      </c>
+      <c r="Z2" s="7" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="AA2" s="7" t="n">
+        <v>771</v>
+      </c>
+      <c r="AB2" s="2" t="n">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPAPSTE01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>RHEL</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 8 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="P3" s="7" t="n">
+        <v>201.6</v>
+      </c>
+      <c r="Q3" s="7" t="n"/>
+      <c r="R3" s="7" t="n"/>
+      <c r="S3" s="7" t="n">
+        <v>111</v>
+      </c>
+      <c r="T3" s="7" t="n">
+        <v>1332</v>
+      </c>
+      <c r="U3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="7" t="n">
+        <v>1244</v>
+      </c>
+      <c r="W3" s="7" t="n">
+        <v>80.33</v>
+      </c>
+      <c r="X3" s="7" t="n">
+        <v>964</v>
+      </c>
+      <c r="Y3" s="7" t="n">
+        <v>876</v>
+      </c>
+      <c r="Z3" s="7" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="AA3" s="7" t="n">
+        <v>771</v>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPAPSRC03</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES23 
+USAEA1PWBWES24</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P4" s="7" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q4" s="7" t="n"/>
+      <c r="R4" s="7" t="n"/>
+      <c r="S4" s="7" t="n">
+        <v>154.83</v>
+      </c>
+      <c r="T4" s="7" t="n">
+        <v>1858</v>
+      </c>
+      <c r="U4" s="7" t="n">
+        <v>806</v>
+      </c>
+      <c r="V4" s="7" t="n">
+        <v>990</v>
+      </c>
+      <c r="W4" s="7" t="n">
+        <v>124.17</v>
+      </c>
+      <c r="X4" s="7" t="n">
+        <v>1490</v>
+      </c>
+      <c r="Y4" s="7" t="n">
+        <v>622</v>
+      </c>
+      <c r="Z4" s="7" t="n">
+        <v>106.33</v>
+      </c>
+      <c r="AA4" s="7" t="n">
+        <v>1276</v>
+      </c>
+      <c r="AB4" s="2" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPAPWFC01</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES25 
+USAEA1PWBWES26</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2019 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="K5" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="P5" s="7" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="Q5" s="7" t="n"/>
+      <c r="R5" s="7" t="n"/>
+      <c r="S5" s="7" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="U5" s="7" t="n">
+        <v>403</v>
+      </c>
+      <c r="V5" s="7" t="n">
+        <v>666</v>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>888</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>441</v>
+      </c>
+      <c r="Z5" s="7" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="AA5" s="7" t="n">
+        <v>749</v>
+      </c>
+      <c r="AB5" s="2" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPWFINT01</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>USAEA1PFSWES09</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2019 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="R6" s="7" t="n">
+        <v>288</v>
+      </c>
+      <c r="S6" s="7" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="T6" s="7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>403</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>666</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>888</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>441</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="AA6" s="7" t="n">
+        <v>749</v>
+      </c>
+      <c r="AB6" s="2" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPWSAPI01</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES35</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="K7" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="R7" s="7" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>154.83</v>
+      </c>
+      <c r="T7" s="7" t="n">
+        <v>1858</v>
+      </c>
+      <c r="U7" s="7" t="n">
+        <v>806</v>
+      </c>
+      <c r="V7" s="7" t="n">
+        <v>990</v>
+      </c>
+      <c r="W7" s="7" t="n">
+        <v>124.17</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>1490</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>622</v>
+      </c>
+      <c r="Z7" s="7" t="n">
+        <v>106.33</v>
+      </c>
+      <c r="AA7" s="7" t="n">
+        <v>1276</v>
+      </c>
+      <c r="AB7" s="2" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPAPWSS03</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES27 
+USAEA1PWBWES28</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="5" t="s">
+      <c r="E8" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="P1" s="3" t="s">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="T8" s="7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>403</v>
+      </c>
+      <c r="V8" s="7" t="n">
+        <v>666</v>
+      </c>
+      <c r="W8" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="X8" s="7" t="n">
+        <v>888</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>441</v>
+      </c>
+      <c r="Z8" s="7" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="AA8" s="7" t="n">
+        <v>749</v>
+      </c>
+      <c r="AB8" s="2" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>PAHWPAPWEF02</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>USAEA1PAPWES34</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q9" s="8" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="R9" s="8" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S9" s="8" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="T9" s="8" t="n">
+        <v>1113</v>
+      </c>
+      <c r="U9" s="8" t="n">
+        <v>403</v>
+      </c>
+      <c r="V9" s="8" t="n">
+        <v>666</v>
+      </c>
+      <c r="W9" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="X9" s="8" t="n">
+        <v>888</v>
+      </c>
+      <c r="Y9" s="8" t="n">
+        <v>441</v>
+      </c>
+      <c r="Z9" s="8" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="AA9" s="8" t="n">
+        <v>749</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="10" ht="30.75" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>PAHWPAPTUI03</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES21 
+USAEA1PWBWES22</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit) [ASG app1 desplegado]</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="M10" s="8" t="n"/>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q10" s="8" t="n"/>
+      <c r="R10" s="8" t="n"/>
+      <c r="S10" s="8" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="T10" s="8" t="n">
+        <v>1113</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>403</v>
+      </c>
+      <c r="V10" s="8" t="n">
+        <v>666</v>
+      </c>
+      <c r="W10" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="X10" s="8" t="n">
+        <v>888</v>
+      </c>
+      <c r="Y10" s="8" t="n">
+        <v>441</v>
+      </c>
+      <c r="Z10" s="8" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="AA10" s="8" t="n">
+        <v>749</v>
+      </c>
+      <c r="AB10" s="2" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>PAHWPCHECS01</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>USAEA1PFSWES08</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2022 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="R11" s="7" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S11" s="7" t="n">
+        <v>154.83</v>
+      </c>
+      <c r="T11" s="7" t="n">
+        <v>1858</v>
+      </c>
+      <c r="U11" s="7" t="n">
+        <v>806</v>
+      </c>
+      <c r="V11" s="7" t="n">
+        <v>990</v>
+      </c>
+      <c r="W11" s="7" t="n">
+        <v>124.17</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>1490</v>
+      </c>
+      <c r="Y11" s="7" t="n">
+        <v>622</v>
+      </c>
+      <c r="Z11" s="7" t="n">
+        <v>106.33</v>
+      </c>
+      <c r="AA11" s="7" t="n">
+        <v>1276</v>
+      </c>
+      <c r="AB11" s="2" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>pahqpapapp02</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>USAEA1PAPWES33</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Windows Server 2019 Standard</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>280</v>
+      </c>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="P12" s="7" t="n">
+        <v>268.8</v>
+      </c>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="7" t="n">
+        <v>89.12</v>
+      </c>
+      <c r="T12" s="7" t="n">
+        <v>1069.42</v>
+      </c>
+      <c r="U12" s="7" t="n">
+        <v>402.96</v>
+      </c>
+      <c r="V12" s="7" t="n">
+        <v>666.46</v>
+      </c>
+      <c r="W12" s="7" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="X12" s="7" t="n">
+        <v>843.76</v>
+      </c>
+      <c r="Y12" s="7" t="n">
+        <v>440.8</v>
+      </c>
+      <c r="Z12" s="7" t="n">
+        <v>58.77</v>
+      </c>
+      <c r="AA12" s="7" t="n">
+        <v>705.27</v>
+      </c>
+      <c r="AB12" s="2" t="n">
+        <v>302.31</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>pahwpapbof01</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04.3 LTS</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>c5a.large</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>c5a.large</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="P13" s="7" t="n">
+        <v>201.6</v>
+      </c>
+      <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="7" t="n"/>
+      <c r="S13" s="7" t="n">
+        <v>56.21</v>
+      </c>
+      <c r="T13" s="7" t="n">
+        <v>674.52</v>
+      </c>
+      <c r="U13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="7" t="n">
+        <v>674.52</v>
+      </c>
+      <c r="W13" s="7" t="n">
+        <v>35.77</v>
+      </c>
+      <c r="X13" s="7" t="n">
+        <v>429.24</v>
+      </c>
+      <c r="Y13" s="7" t="n">
+        <v>429.24</v>
+      </c>
+      <c r="Z13" s="7" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="AA13" s="7" t="n">
+        <v>289.08</v>
+      </c>
+      <c r="AB13" s="2" t="n">
+        <v>289.08</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>RDS produccion (multiaz1)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>SQL Server - Standard</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>SQL Server Standard Edition 15.x (Multi-AZ, license-included)</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>db.r6i.4xlarge</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>db.r6i.4xlarge</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>1700</v>
+      </c>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="n">
+        <v>272</v>
+      </c>
+      <c r="P14" s="7" t="n">
+        <v>3264</v>
+      </c>
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
+      <c r="S14" s="7" t="n">
+        <v>8876.799999999999</v>
+      </c>
+      <c r="T14" s="7" t="n">
+        <v>106521.6</v>
+      </c>
+      <c r="U14" s="7" t="n">
+        <v>54382.08</v>
+      </c>
+      <c r="V14" s="7" t="n">
+        <v>52139.52</v>
+      </c>
+      <c r="W14" s="7" t="n">
+        <v>8388.58</v>
+      </c>
+      <c r="X14" s="7" t="n">
+        <v>100662.91</v>
+      </c>
+      <c r="Y14" s="7" t="n"/>
+      <c r="Z14" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA14" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>RDS procesos (standalone1)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>SQL Server - Standard</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>SQL Server Standard Edition 15.x (Single-AZ, license-included)</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>db.r6i.2xlarge</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>db.r6i.2xlarge</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>232</v>
+      </c>
+      <c r="P15" s="7" t="n">
+        <v>2784</v>
+      </c>
+      <c r="Q15" s="7" t="n"/>
+      <c r="R15" s="7" t="n"/>
+      <c r="S15" s="7" t="n">
+        <v>2219.2</v>
+      </c>
+      <c r="T15" s="7" t="n">
+        <v>26630.4</v>
+      </c>
+      <c r="U15" s="7" t="n">
+        <v>13595.52</v>
+      </c>
+      <c r="V15" s="7" t="n">
+        <v>13034.88</v>
+      </c>
+      <c r="W15" s="7" t="n">
+        <v>2097.14</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>25165.73</v>
+      </c>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA15" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>FSx Windows (intelisrcpa-prd)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Windows (FSx)</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>FSx Windows File Server Single-AZ SSD (64 MBps, backup 30d)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>FSx SINGLE_AZ_1</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>FSx SINGLE_AZ_1</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="Q1" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" s="3" t="s">
+      <c r="P16" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="7" t="n"/>
+      <c r="S16" s="7" t="n">
+        <v>140.8</v>
+      </c>
+      <c r="T16" s="7" t="n">
+        <v>1689.6</v>
+      </c>
+      <c r="U16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="7" t="n">
+        <v>1689.6</v>
+      </c>
+      <c r="W16" s="7" t="n"/>
+      <c r="X16" s="7" t="n"/>
+      <c r="Y16" s="7" t="n"/>
+      <c r="Z16" s="7" t="n"/>
+      <c r="AA16" s="7" t="n"/>
+      <c r="AB16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>AMI Builder (temporal)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (AMI Builder - temporal)</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>m5.large</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>m5.large</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="P17" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q17" s="7" t="n"/>
+      <c r="R17" s="7" t="n"/>
+      <c r="S17" s="7" t="n">
+        <v>137.24</v>
+      </c>
+      <c r="T17" s="7" t="n">
+        <v>1646.88</v>
+      </c>
+      <c r="U17" s="7" t="n">
+        <v>805.92</v>
+      </c>
+      <c r="V17" s="7" t="n">
+        <v>840.96</v>
+      </c>
+      <c r="W17" s="7" t="n">
+        <v>110.96</v>
+      </c>
+      <c r="X17" s="7" t="n">
+        <v>1331.52</v>
+      </c>
+      <c r="Y17" s="7" t="n">
+        <v>525.6</v>
+      </c>
+      <c r="Z17" s="7" t="n">
+        <v>97.09</v>
+      </c>
+      <c r="AA17" s="7" t="n">
+        <v>1165.08</v>
+      </c>
+      <c r="AB17" s="2" t="n">
+        <v>359.16</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>DMS replication (poc)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="W1" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB1" s="6" t="s">
-        <v>20</v>
-      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>DMS</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>DMS c5.2xlarge Single-AZ (engine 3.6.1)</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>dms.c5.2xlarge</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>dms.c5.2xlarge</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="P18" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="Q18" s="7" t="n"/>
+      <c r="R18" s="7" t="n"/>
+      <c r="S18" s="7" t="n">
+        <v>347.48</v>
+      </c>
+      <c r="T18" s="7" t="n">
+        <v>4169.76</v>
+      </c>
+      <c r="U18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="7" t="n">
+        <v>4169.76</v>
+      </c>
+      <c r="W18" s="7" t="n"/>
+      <c r="X18" s="7" t="n"/>
+      <c r="Y18" s="7" t="n"/>
+      <c r="Z18" s="7" t="n"/>
+      <c r="AA18" s="7" t="n"/>
+      <c r="AB18" s="2" t="n"/>
     </row>
-    <row r="2" spans="1:28" ht="15.75">
-      <c r="A2" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="7">
-        <v>4</v>
-      </c>
-      <c r="E2" s="7">
-        <v>16</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" s="7">
-        <v>2</v>
-      </c>
-      <c r="K2" s="7">
-        <v>16</v>
-      </c>
-      <c r="L2" s="7">
-        <v>520</v>
-      </c>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7">
-        <v>499.2</v>
-      </c>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-      <c r="S2" s="7"/>
-      <c r="T2" s="7">
-        <v>1332</v>
-      </c>
-      <c r="U2" s="7">
-        <v>0</v>
-      </c>
-      <c r="V2" s="7">
-        <v>1244</v>
-      </c>
-      <c r="W2" s="7"/>
-      <c r="X2" s="7">
-        <v>964</v>
-      </c>
-      <c r="Y2" s="7">
-        <v>876</v>
-      </c>
-      <c r="Z2" s="7"/>
-      <c r="AA2" s="7">
-        <v>771</v>
-      </c>
-      <c r="AB2" s="2">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" ht="15.75">
-      <c r="A3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="7">
-        <v>4</v>
-      </c>
-      <c r="E3" s="7">
-        <v>16</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="7">
-        <v>2</v>
-      </c>
-      <c r="K3" s="7">
-        <v>16</v>
-      </c>
-      <c r="L3" s="7">
-        <v>210</v>
-      </c>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7">
-        <v>201.6</v>
-      </c>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="7">
-        <v>1332</v>
-      </c>
-      <c r="U3" s="7">
-        <v>0</v>
-      </c>
-      <c r="V3" s="7">
-        <v>1244</v>
-      </c>
-      <c r="W3" s="7"/>
-      <c r="X3" s="7">
-        <v>964</v>
-      </c>
-      <c r="Y3" s="7">
-        <v>876</v>
-      </c>
-      <c r="Z3" s="7"/>
-      <c r="AA3" s="7">
-        <v>771</v>
-      </c>
-      <c r="AB3" s="2">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" ht="30" customHeight="1">
-      <c r="A4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="7">
-        <v>4</v>
-      </c>
-      <c r="E4" s="7">
-        <v>16</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="7">
-        <v>2</v>
-      </c>
-      <c r="K4" s="7">
-        <v>16</v>
-      </c>
-      <c r="L4" s="7">
-        <v>120</v>
-      </c>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7">
-        <v>115.2</v>
-      </c>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7">
-        <v>1858</v>
-      </c>
-      <c r="U4" s="7">
-        <v>806</v>
-      </c>
-      <c r="V4" s="7">
-        <v>990</v>
-      </c>
-      <c r="W4" s="7"/>
-      <c r="X4" s="7">
-        <v>1490</v>
-      </c>
-      <c r="Y4" s="7">
-        <v>622</v>
-      </c>
-      <c r="Z4" s="7"/>
-      <c r="AA4" s="7">
-        <v>1276</v>
-      </c>
-      <c r="AB4" s="2">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" ht="30" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="7">
-        <v>4</v>
-      </c>
-      <c r="E5" s="7">
-        <v>8</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" s="7">
-        <v>1</v>
-      </c>
-      <c r="K5" s="7">
-        <v>8</v>
-      </c>
-      <c r="L5" s="7">
-        <v>80</v>
-      </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7">
-        <v>76.8</v>
-      </c>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="7"/>
-      <c r="T5" s="7">
-        <v>1113</v>
-      </c>
-      <c r="U5" s="7">
-        <v>403</v>
-      </c>
-      <c r="V5" s="7">
-        <v>666</v>
-      </c>
-      <c r="W5" s="7"/>
-      <c r="X5" s="7">
-        <v>888</v>
-      </c>
-      <c r="Y5" s="7">
-        <v>441</v>
-      </c>
-      <c r="Z5" s="7"/>
-      <c r="AA5" s="7">
-        <v>749</v>
-      </c>
-      <c r="AB5" s="2">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" ht="15.75">
-      <c r="A6" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="7">
-        <v>4</v>
-      </c>
-      <c r="E6" s="7">
-        <v>8</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="7">
-        <v>1</v>
-      </c>
-      <c r="K6" s="7">
-        <v>8</v>
-      </c>
-      <c r="L6" s="7">
-        <v>80</v>
-      </c>
-      <c r="M6" s="7">
-        <v>300</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7">
-        <v>76.8</v>
-      </c>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="S6" s="7"/>
-      <c r="T6" s="7">
-        <v>1113</v>
-      </c>
-      <c r="U6" s="7">
-        <v>403</v>
-      </c>
-      <c r="V6" s="7">
-        <v>666</v>
-      </c>
-      <c r="W6" s="7"/>
-      <c r="X6" s="7">
-        <v>888</v>
-      </c>
-      <c r="Y6" s="7">
-        <v>441</v>
-      </c>
-      <c r="Z6" s="7"/>
-      <c r="AA6" s="7">
-        <v>749</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" ht="15.75">
-      <c r="A7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="7">
-        <v>4</v>
-      </c>
-      <c r="E7" s="7">
-        <v>16</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J7" s="7">
-        <v>2</v>
-      </c>
-      <c r="K7" s="7">
-        <v>16</v>
-      </c>
-      <c r="L7" s="7">
-        <v>120</v>
-      </c>
-      <c r="M7" s="7">
-        <v>90</v>
-      </c>
-      <c r="N7" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7">
-        <v>115.2</v>
-      </c>
-      <c r="Q7" s="7"/>
-      <c r="R7" s="7"/>
-      <c r="S7" s="7"/>
-      <c r="T7" s="7">
-        <v>1858</v>
-      </c>
-      <c r="U7" s="7">
-        <v>806</v>
-      </c>
-      <c r="V7" s="7">
-        <v>990</v>
-      </c>
-      <c r="W7" s="7"/>
-      <c r="X7" s="7">
-        <v>1490</v>
-      </c>
-      <c r="Y7" s="7">
-        <v>622</v>
-      </c>
-      <c r="Z7" s="7"/>
-      <c r="AA7" s="7">
-        <v>1276</v>
-      </c>
-      <c r="AB7" s="2">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" ht="30" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="7">
-        <v>4</v>
-      </c>
-      <c r="E8" s="7">
-        <v>8</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="7">
-        <v>1</v>
-      </c>
-      <c r="K8" s="7">
-        <v>8</v>
-      </c>
-      <c r="L8" s="7">
-        <v>120</v>
-      </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7">
-        <v>115.2</v>
-      </c>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="7">
-        <v>1113</v>
-      </c>
-      <c r="U8" s="7">
-        <v>403</v>
-      </c>
-      <c r="V8" s="7">
-        <v>666</v>
-      </c>
-      <c r="W8" s="7"/>
-      <c r="X8" s="7">
-        <v>888</v>
-      </c>
-      <c r="Y8" s="7">
-        <v>441</v>
-      </c>
-      <c r="Z8" s="7"/>
-      <c r="AA8" s="7">
-        <v>749</v>
-      </c>
-      <c r="AB8" s="2">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" ht="15.75">
-      <c r="A9" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="8">
-        <v>4</v>
-      </c>
-      <c r="E9" s="8">
-        <v>8</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J9" s="8">
-        <v>1</v>
-      </c>
-      <c r="K9" s="8">
-        <v>8</v>
-      </c>
-      <c r="L9" s="8">
-        <v>120</v>
-      </c>
-      <c r="M9" s="8">
-        <v>90</v>
-      </c>
-      <c r="N9" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8">
-        <v>115.2</v>
-      </c>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="8"/>
-      <c r="S9" s="8"/>
-      <c r="T9" s="8">
-        <v>1113</v>
-      </c>
-      <c r="U9" s="8">
-        <v>403</v>
-      </c>
-      <c r="V9" s="8">
-        <v>666</v>
-      </c>
-      <c r="W9" s="8"/>
-      <c r="X9" s="8">
-        <v>888</v>
-      </c>
-      <c r="Y9" s="8">
-        <v>441</v>
-      </c>
-      <c r="Z9" s="8"/>
-      <c r="AA9" s="8">
-        <v>749</v>
-      </c>
-      <c r="AB9" s="2">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" ht="30.75">
-      <c r="A10" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="8">
-        <v>4</v>
-      </c>
-      <c r="E10" s="8">
-        <v>8</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J10" s="8">
-        <v>1</v>
-      </c>
-      <c r="K10" s="8">
-        <v>8</v>
-      </c>
-      <c r="L10" s="8">
-        <v>120</v>
-      </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8">
-        <v>115.2</v>
-      </c>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8">
-        <v>1113</v>
-      </c>
-      <c r="U10" s="8">
-        <v>403</v>
-      </c>
-      <c r="V10" s="8">
-        <v>666</v>
-      </c>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8">
-        <v>888</v>
-      </c>
-      <c r="Y10" s="8">
-        <v>441</v>
-      </c>
-      <c r="Z10" s="8"/>
-      <c r="AA10" s="8">
-        <v>749</v>
-      </c>
-      <c r="AB10" s="2">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" ht="30" customHeight="1">
-      <c r="A11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="7">
-        <v>4</v>
-      </c>
-      <c r="E11" s="7">
-        <v>16</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J11" s="7">
-        <v>2</v>
-      </c>
-      <c r="K11" s="7">
-        <v>16</v>
-      </c>
-      <c r="L11" s="7">
-        <v>120</v>
-      </c>
-      <c r="M11" s="7">
-        <v>90</v>
-      </c>
-      <c r="N11" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7">
-        <v>115.2</v>
-      </c>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
-      <c r="S11" s="7"/>
-      <c r="T11" s="7">
-        <v>1858</v>
-      </c>
-      <c r="U11" s="7">
-        <v>806</v>
-      </c>
-      <c r="V11" s="7">
-        <v>990</v>
-      </c>
-      <c r="W11" s="7"/>
-      <c r="X11" s="7">
-        <v>1490</v>
-      </c>
-      <c r="Y11" s="7">
-        <v>622</v>
-      </c>
-      <c r="Z11" s="7"/>
-      <c r="AA11" s="7">
-        <v>1276</v>
-      </c>
-      <c r="AB11" s="2">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" ht="15.75">
-      <c r="A12" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="7">
-        <v>4</v>
-      </c>
-      <c r="E12" s="7">
-        <v>8</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J12" s="7">
-        <v>4</v>
-      </c>
-      <c r="K12" s="7">
-        <v>8</v>
-      </c>
-      <c r="L12" s="7">
-        <v>280</v>
-      </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7">
-        <v>268.8</v>
-      </c>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
-      <c r="S12" s="7"/>
-      <c r="T12" s="7">
-        <v>1069.42</v>
-      </c>
-      <c r="U12" s="7">
-        <v>402.96</v>
-      </c>
-      <c r="V12" s="7">
-        <v>666.46</v>
-      </c>
-      <c r="W12" s="7"/>
-      <c r="X12" s="7">
-        <v>843.76</v>
-      </c>
-      <c r="Y12" s="7">
-        <v>440.8</v>
-      </c>
-      <c r="Z12" s="7"/>
-      <c r="AA12" s="7">
-        <v>705.27</v>
-      </c>
-      <c r="AB12" s="2">
-        <v>302.31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" ht="15.75">
-      <c r="A13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="7">
-        <v>4</v>
-      </c>
-      <c r="E13" s="7">
-        <v>2</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="J13" s="7">
-        <v>2</v>
-      </c>
-      <c r="K13" s="7">
-        <v>4</v>
-      </c>
-      <c r="L13" s="7">
-        <v>210</v>
-      </c>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7">
-        <v>201.6</v>
-      </c>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
-      <c r="S13" s="7"/>
-      <c r="T13" s="7">
-        <v>674.52</v>
-      </c>
-      <c r="U13" s="7">
-        <v>0</v>
-      </c>
-      <c r="V13" s="7">
-        <v>674.52</v>
-      </c>
-      <c r="W13" s="7"/>
-      <c r="X13" s="7">
-        <v>429.24</v>
-      </c>
-      <c r="Y13" s="7">
-        <v>429.24</v>
-      </c>
-      <c r="Z13" s="7"/>
-      <c r="AA13" s="7">
-        <v>289.08</v>
-      </c>
-      <c r="AB13" s="2">
-        <v>289.08</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" ht="15.75">
-      <c r="A14" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="7">
-        <v>16</v>
-      </c>
-      <c r="E14" s="7">
-        <v>128</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J14" s="7">
-        <v>16</v>
-      </c>
-      <c r="K14" s="7">
-        <v>128</v>
-      </c>
-      <c r="L14" s="7">
-        <v>1700</v>
-      </c>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7">
-        <v>3264</v>
-      </c>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
-      <c r="S14" s="7"/>
-      <c r="T14" s="7">
-        <v>106521.60000000001</v>
-      </c>
-      <c r="U14" s="7">
-        <v>54382.080000000002</v>
-      </c>
-      <c r="V14" s="7">
-        <v>52139.519999999997</v>
-      </c>
-      <c r="W14" s="7"/>
-      <c r="X14" s="7">
-        <v>100662.91</v>
-      </c>
-      <c r="Y14" s="7"/>
-      <c r="Z14" s="7"/>
-      <c r="AA14" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB14" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" ht="15.75">
-      <c r="A15" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="7">
-        <v>8</v>
-      </c>
-      <c r="E15" s="7">
-        <v>64</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="J15" s="7">
-        <v>8</v>
-      </c>
-      <c r="K15" s="7">
-        <v>64</v>
-      </c>
-      <c r="L15" s="7">
-        <v>2900</v>
-      </c>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7">
-        <v>2784</v>
-      </c>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="7">
-        <v>26630.400000000001</v>
-      </c>
-      <c r="U15" s="7">
-        <v>13595.52</v>
-      </c>
-      <c r="V15" s="7">
-        <v>13034.88</v>
-      </c>
-      <c r="W15" s="7"/>
-      <c r="X15" s="7">
-        <v>25165.73</v>
-      </c>
-      <c r="Y15" s="7"/>
-      <c r="Z15" s="7"/>
-      <c r="AA15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB15" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" ht="15.75">
-      <c r="A16" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7">
-        <v>100</v>
-      </c>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7">
-        <v>156</v>
-      </c>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
-      <c r="S16" s="7"/>
-      <c r="T16" s="7">
-        <v>1689.6</v>
-      </c>
-      <c r="U16" s="7">
-        <v>0</v>
-      </c>
-      <c r="V16" s="7">
-        <v>1689.6</v>
-      </c>
-      <c r="W16" s="7"/>
-      <c r="X16" s="7"/>
-      <c r="Y16" s="7"/>
-      <c r="Z16" s="7"/>
-      <c r="AA16" s="7"/>
-      <c r="AB16" s="2"/>
-    </row>
-    <row r="17" spans="1:28" ht="15.75">
-      <c r="A17" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="7">
-        <v>2</v>
-      </c>
-      <c r="E17" s="7">
-        <v>8</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J17" s="7">
-        <v>2</v>
-      </c>
-      <c r="K17" s="7">
-        <v>8</v>
-      </c>
-      <c r="L17" s="7">
-        <v>100</v>
-      </c>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7">
-        <v>96</v>
-      </c>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7">
-        <v>1646.88</v>
-      </c>
-      <c r="U17" s="7">
-        <v>805.92</v>
-      </c>
-      <c r="V17" s="7">
-        <v>840.96</v>
-      </c>
-      <c r="W17" s="7"/>
-      <c r="X17" s="7">
-        <v>1331.52</v>
-      </c>
-      <c r="Y17" s="7">
-        <v>525.6</v>
-      </c>
-      <c r="Z17" s="7"/>
-      <c r="AA17" s="7">
-        <v>1165.08</v>
-      </c>
-      <c r="AB17" s="2">
-        <v>359.16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" ht="15.75">
-      <c r="A18" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="7">
-        <v>8</v>
-      </c>
-      <c r="E18" s="7">
-        <v>16</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="J18" s="7">
-        <v>8</v>
-      </c>
-      <c r="K18" s="7">
-        <v>16</v>
-      </c>
-      <c r="L18" s="7">
-        <v>50</v>
-      </c>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7">
-        <v>69</v>
-      </c>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-      <c r="S18" s="7"/>
-      <c r="T18" s="7">
-        <v>4169.76</v>
-      </c>
-      <c r="U18" s="7">
-        <v>0</v>
-      </c>
-      <c r="V18" s="7">
-        <v>4169.76</v>
-      </c>
-      <c r="W18" s="7"/>
-      <c r="X18" s="7"/>
-      <c r="Y18" s="7"/>
-      <c r="Z18" s="7"/>
-      <c r="AA18" s="7"/>
-      <c r="AB18" s="2"/>
-    </row>
-    <row r="19" spans="1:28"/>
-    <row r="20" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="21" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="22" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:28" ht="15.75" customHeight="1"/>
+    <row r="20" ht="15.75" customHeight="1"/>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
feat: add ALB, ASG lifecycle, S3, Secrets Manager and CloudWatch to prod TCO
</commit_message>
<xml_diff>
--- a/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
+++ b/Ambiente Productivo/Lift-and-Shift - 18 Servers/analysis_TCO.xlsx
@@ -1,482 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C29652e\projects\Assessment\Assessment\Ambiente Productivo\Lift-and-Shift - 18 Servers\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4D3653-1FE1-4B0A-8EBF-947BD99B87BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" r:id="rId1"/>
-    <sheet name="Glossary" sheetId="2" r:id="rId2"/>
-    <sheet name="Shared Tenancy Analysis" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Tenancy Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={5D300EF5-99F3-47D0-9E4E-574991756B1B}</author>
-    <author>tc={9766D75B-3A6E-45AA-8036-B209058EFE63}</author>
-    <author>tc={7CBE9C47-E890-4965-BEAF-A26D0A421EE9}</author>
-    <author>tc={C1EC95D0-3745-42C2-8CCD-73E88C66B3F6}</author>
-    <author>tc={765B32F2-5618-4970-AFAB-880B3045A5ED}</author>
-    <author>tc={A5E9C293-0AAB-4608-A30C-900615DA4063}</author>
-  </authors>
-  <commentList>
-    <comment ref="Z14" authorId="0" shapeId="0" xr:uid="{5D300EF5-99F3-47D0-9E4E-574991756B1B}">
-      <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    All upfront</t>
-      </text>
-    </comment>
-    <comment ref="AA14" authorId="1" shapeId="0" xr:uid="{9766D75B-3A6E-45AA-8036-B209058EFE63}">
-      <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    All upfront</t>
-      </text>
-    </comment>
-    <comment ref="Z15" authorId="2" shapeId="0" xr:uid="{7CBE9C47-E890-4965-BEAF-A26D0A421EE9}">
-      <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    All upfront</t>
-      </text>
-    </comment>
-    <comment ref="AA15" authorId="3" shapeId="0" xr:uid="{C1EC95D0-3745-42C2-8CCD-73E88C66B3F6}">
-      <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    All upfront</t>
-      </text>
-    </comment>
-    <comment ref="O16" authorId="4" shapeId="0" xr:uid="{765B32F2-5618-4970-AFAB-880B3045A5ED}">
-      <text>
-        <t xml:space="preserve">[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    Storage + throughput  </t>
-      </text>
-    </comment>
-    <comment ref="S16" authorId="5" shapeId="0" xr:uid="{A5E9C293-0AAB-4608-A30C-900615DA4063}">
-      <text>
-        <t xml:space="preserve">[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    Storage + throughput  
-Facturado
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="113">
-  <si>
-    <t>Host Name Onpremise</t>
-  </si>
-  <si>
-    <t>EC2 Name</t>
-  </si>
-  <si>
-    <t>Enviroment</t>
-  </si>
-  <si>
-    <t>Number of CPUs</t>
-  </si>
-  <si>
-    <t>RAM (GB)</t>
-  </si>
-  <si>
-    <t>Operation System Type</t>
-  </si>
-  <si>
-    <t>Operation System Name</t>
-  </si>
-  <si>
-    <t>AWS Instance Recommended</t>
-  </si>
-  <si>
-    <t>AWS Instance Deploy</t>
-  </si>
-  <si>
-    <t>AWS Total Cores</t>
-  </si>
-  <si>
-    <t>AWS RAM (GB)</t>
-  </si>
-  <si>
-    <t>EBS Size (GB)</t>
-  </si>
-  <si>
-    <t>EBS Additional Size (GB)</t>
-  </si>
-  <si>
-    <t>AWS Region</t>
-  </si>
-  <si>
-    <t>Monthly Root EBS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr EBS Cost</t>
-  </si>
-  <si>
-    <t>Monthly Additional EBS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr Additional EBS Cost</t>
-  </si>
-  <si>
-    <t>Monthly  On-Demand Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized On-Demand Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized License Only Cost</t>
-  </si>
-  <si>
-    <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
-  </si>
-  <si>
-    <t>Monthly 1 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
-  </si>
-  <si>
-    <t>Monthly 3 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
-  </si>
-  <si>
-    <t>Annualized 3 Yr NURI Total EC2 Cost</t>
-  </si>
-  <si>
-    <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
-  </si>
-  <si>
-    <t>PAHWPAPSTS01</t>
-  </si>
-  <si>
-    <t>PROD</t>
-  </si>
-  <si>
-    <t>RHEL</t>
-  </si>
-  <si>
-    <t>Red Hat Enterprise Linux 8 (64-bit)</t>
-  </si>
-  <si>
-    <t>r5a.large</t>
-  </si>
-  <si>
-    <t>US East (N. Virginia)</t>
-  </si>
-  <si>
-    <t>PAHWPAPSTE01</t>
-  </si>
-  <si>
-    <t>PAHWPAPSRC03</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES23 
-USAEA1PWBWES24</t>
-  </si>
-  <si>
-    <t>Windows</t>
-  </si>
-  <si>
-    <t>PAHWPAPWFC01</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES25 
-USAEA1PWBWES26</t>
-  </si>
-  <si>
-    <t>r7a.medium</t>
-  </si>
-  <si>
-    <t>PAHWPWFINT01</t>
-  </si>
-  <si>
-    <t>USAEA1PFSWES09</t>
-  </si>
-  <si>
-    <t>PAHWPWSAPI01</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES35</t>
-  </si>
-  <si>
-    <t>PAHWPAPWSS03</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES27 
-USAEA1PWBWES28</t>
-  </si>
-  <si>
-    <t>PAHWPAPWEF02</t>
-  </si>
-  <si>
-    <t>USAEA1PAPWES34</t>
-  </si>
-  <si>
-    <t>PAHWPAPTUI03</t>
-  </si>
-  <si>
-    <t>USAEA1PWBWES21 
-USAEA1PWBWES22</t>
-  </si>
-  <si>
-    <t>PAHWPCHECS01</t>
-  </si>
-  <si>
-    <t>USAEA1PFSWES08</t>
-  </si>
-  <si>
-    <t>pahqpapapp02</t>
-  </si>
-  <si>
-    <t>USAEA1PAPWES33</t>
-  </si>
-  <si>
-    <t>pahwpapbof01</t>
-  </si>
-  <si>
-    <t>Linux</t>
-  </si>
-  <si>
-    <t>c5a.large</t>
-  </si>
-  <si>
-    <t>RDS produccion (multiaz1)</t>
-  </si>
-  <si>
-    <t>SQL Server - Standard</t>
-  </si>
-  <si>
-    <t>SQL Server Standard Edition 15.x (Multi-AZ, license-included)</t>
-  </si>
-  <si>
-    <t>db.r6i.4xlarge</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>RDS procesos (standalone1)</t>
-  </si>
-  <si>
-    <t>SQL Server Standard Edition 15.x (Single-AZ, license-included)</t>
-  </si>
-  <si>
-    <t>db.r6i.2xlarge</t>
-  </si>
-  <si>
-    <t>FSx Windows (intelisrcpa-prd)</t>
-  </si>
-  <si>
-    <t>Windows (FSx)</t>
-  </si>
-  <si>
-    <t>FSx Windows File Server Single-AZ SSD (64 MBps, backup 30d)</t>
-  </si>
-  <si>
-    <t>FSx SINGLE_AZ_1</t>
-  </si>
-  <si>
-    <t>AMI Builder (temporal)</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2025 (AMI Builder - temporal)</t>
-  </si>
-  <si>
-    <t>m5.large</t>
-  </si>
-  <si>
-    <t>DMS</t>
-  </si>
-  <si>
-    <t>DMS c5.2xlarge Single-AZ (engine 3.6.1)</t>
-  </si>
-  <si>
-    <t>dms.c5.2xlarge</t>
-  </si>
-  <si>
-    <t>This file contains an export of AWS Transform Assessment results for Production Environment (InteliSrcPA).</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Glossary</t>
-  </si>
-  <si>
-    <t>Column-by-column definitions and descriptions for all data fields.</t>
-  </si>
-  <si>
-    <t>Shared Tenancy Analysis</t>
-  </si>
-  <si>
-    <t>Lists servers that can run on shared hardware infrastructure in AWS.</t>
-  </si>
-  <si>
-    <t>Attribute Name</t>
-  </si>
-  <si>
-    <t>Name assigned to the server on-premise</t>
-  </si>
-  <si>
-    <t>Name for the EC2 instance in AWS</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Production/Development/Test environment designation</t>
-  </si>
-  <si>
-    <t>Count of virtual processors</t>
-  </si>
-  <si>
-    <t>Total memory capacity in gigabytes</t>
-  </si>
-  <si>
-    <t>Category of operating system</t>
-  </si>
-  <si>
-    <t>Specific OS version/distribution</t>
-  </si>
-  <si>
-    <t>Recommended AWS instance type by assessment tool</t>
-  </si>
-  <si>
-    <t>Instance type to be deployed</t>
-  </si>
-  <si>
-    <t>Total cores in recommended EC2 instance</t>
-  </si>
-  <si>
-    <t>Memory in recommended instance in GB</t>
-  </si>
-  <si>
-    <t>Root volume EBS storage size in GB</t>
-  </si>
-  <si>
-    <t>EBS Size (GB) Additional</t>
-  </si>
-  <si>
-    <t>Additional EBS volumes in GB</t>
-  </si>
-  <si>
-    <t>Target AWS geographic region</t>
-  </si>
-  <si>
-    <t>Yearly EBS storage cost</t>
-  </si>
-  <si>
-    <t>Yearly total cost using on-demand pricing</t>
-  </si>
-  <si>
-    <t>Yearly licensing costs</t>
-  </si>
-  <si>
-    <t>Yearly compute costs at on-demand rates</t>
-  </si>
-  <si>
-    <t>Total yearly cost with 1-year RI no upfront</t>
-  </si>
-  <si>
-    <t>Compute-only yearly cost with 1-year RI</t>
-  </si>
-  <si>
-    <t>Total yearly cost with 3-year RI no upfront</t>
-  </si>
-  <si>
-    <t>Compute-only yearly cost with 3-year RI</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2025 (64-bit)</t>
-  </si>
-  <si>
-    <t>Microsoft Windows Server 2025 (64-bit) [ASG app1 desplegado]</t>
-  </si>
-  <si>
-    <t>Windows Server 2025 Standard</t>
-  </si>
-  <si>
-    <t>Ubuntu 22.04.3 LTS TBD</t>
-  </si>
-  <si>
-    <t>DMS replication</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Amazon Ember"/>
+      <b val="1"/>
+      <color theme="0"/>
       <sz val="12"/>
-      <color theme="0"/>
-      <name val="Amazon Ember"/>
     </font>
     <font>
+      <name val="Amazon Ember"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Amazon Ember"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -532,47 +101,165 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Sepulveda.ext, Javier" id="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" userId="S::Javier.Sepulveda.ext@experian.com::a98f7e8a-e365-4515-8010-0c968fd6c46a" providerId="AD"/>
-</personList>
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>tc={5D300EF5-99F3-47D0-9E4E-574991756B1B}</author>
+    <author>tc={9766D75B-3A6E-45AA-8036-B209058EFE63}</author>
+    <author>tc={7CBE9C47-E890-4965-BEAF-A26D0A421EE9}</author>
+    <author>tc={C1EC95D0-3745-42C2-8CCD-73E88C66B3F6}</author>
+    <author>tc={765B32F2-5618-4970-AFAB-880B3045A5ED}</author>
+    <author>tc={A5E9C293-0AAB-4608-A30C-900615DA4063}</author>
+  </authors>
+  <commentList>
+    <comment ref="Z14" authorId="0" shapeId="0">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    All upfront</t>
+      </text>
+    </comment>
+    <comment ref="AA14" authorId="1" shapeId="0">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    All upfront</t>
+      </text>
+    </comment>
+    <comment ref="Z15" authorId="2" shapeId="0">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    All upfront</t>
+      </text>
+    </comment>
+    <comment ref="AA15" authorId="3" shapeId="0">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    All upfront</t>
+      </text>
+    </comment>
+    <comment ref="O16" authorId="4" shapeId="0">
+      <text>
+        <t xml:space="preserve">[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Storage + throughput  </t>
+      </text>
+    </comment>
+    <comment ref="S16" authorId="5" shapeId="0">
+      <text>
+        <t xml:space="preserve">[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Storage + throughput  
+Facturado
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -771,66 +458,59 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="Z14" dT="2026-09-01T17:56:19.42" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{5D300EF5-99F3-47D0-9E4E-574991756B1B}">
-    <text>All upfront</text>
-  </threadedComment>
-  <threadedComment ref="AA14" dT="2026-09-01T17:56:24.62" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{9766D75B-3A6E-45AA-8036-B209058EFE63}">
-    <text>All upfront</text>
-  </threadedComment>
-  <threadedComment ref="Z15" dT="2026-09-01T18:00:49.50" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{7CBE9C47-E890-4965-BEAF-A26D0A421EE9}">
-    <text>All upfront</text>
-  </threadedComment>
-  <threadedComment ref="AA15" dT="2026-09-01T18:01:11.78" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{C1EC95D0-3745-42C2-8CCD-73E88C66B3F6}">
-    <text>All upfront</text>
-  </threadedComment>
-  <threadedComment ref="O16" dT="2026-09-01T18:07:11.80" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{765B32F2-5618-4970-AFAB-880B3045A5ED}">
-    <text xml:space="preserve">Storage + throughput  </text>
-  </threadedComment>
-  <threadedComment ref="S16" dT="2026-09-01T18:08:50.11" personId="{9A2084DB-0935-46EE-9D2A-62DAD6A79022}" id="{A5E9C293-0AAB-4608-A30C-900615DA4063}">
-    <text xml:space="preserve">Storage + throughput  
-Facturado
-</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="8.7109375" customWidth="1"/>
+    <col width="8.7109375" customWidth="1" min="1" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>76</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>This file contains an export of AWS Transform Assessment results for Production Environment (InteliSrcPA).</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>78</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>80</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Glossary</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Column-by-column definitions and descriptions for all data fields.</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>82</v>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Shared Tenancy Analysis</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Lists servers that can run on shared hardware infrastructure in AWS.</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1820,210 +1500,308 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="26" width="8.7109375" customWidth="1"/>
+    <col width="8.7109375" customWidth="1" min="1" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>78</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Attribute Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>81</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Shared Tenancy Analysis</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>84</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Host Name Onpremise</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Name assigned to the server on-premise</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>85</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EC2 Name</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Name for the EC2 instance in AWS</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>87</v>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Production/Development/Test environment designation</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>88</v>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Number of CPUs</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Count of virtual processors</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>89</v>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>RAM (GB)</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Total memory capacity in gigabytes</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>90</v>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Operation System Type</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Category of operating system</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>91</v>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Operation System Name</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Specific OS version/distribution</t>
+        </is>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>92</v>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>AWS Instance Recommended</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Recommended AWS instance type by assessment tool</t>
+        </is>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>93</v>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>AWS Instance Deploy</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Instance type to be deployed</t>
+        </is>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>94</v>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>AWS Total Cores</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Total cores in recommended EC2 instance</t>
+        </is>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>95</v>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>AWS RAM (GB)</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Memory in recommended instance in GB</t>
+        </is>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>96</v>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>EBS Size (GB)</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Root volume EBS storage size in GB</t>
+        </is>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>98</v>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>EBS Size (GB) Additional</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Additional EBS volumes in GB</t>
+        </is>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>99</v>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>AWS Region</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Target AWS geographic region</t>
+        </is>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>100</v>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr EBS Cost</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Yearly EBS storage cost</t>
+        </is>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>101</v>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Yearly total cost using on-demand pricing</t>
+        </is>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>102</v>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Annualized License Only Cost</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Yearly licensing costs</t>
+        </is>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>103</v>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Yearly compute costs at on-demand rates</t>
+        </is>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>104</v>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Total yearly cost with 1-year RI no upfront</t>
+        </is>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A22" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>105</v>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Compute-only yearly cost with 1-year RI</t>
+        </is>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>106</v>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI Total EC2 Cost</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Total yearly cost with 3-year RI no upfront</t>
+        </is>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A24" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>107</v>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Compute-only yearly cost with 3-year RI</t>
+        </is>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:2" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2999,1532 +2777,2162 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AB999"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="67.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23" customWidth="1"/>
-    <col min="15" max="15" width="27.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26" customWidth="1"/>
-    <col min="17" max="17" width="33.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="48.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="51.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="30" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="40" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="79.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="40" customWidth="1"/>
-    <col min="25" max="25" width="40" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="79.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="37" customWidth="1"/>
-    <col min="28" max="28" width="40" hidden="1" customWidth="1"/>
-    <col min="29" max="32" width="8.7109375" customWidth="1"/>
+    <col width="31.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="48.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="27.140625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="67.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="34.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="25" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="19.85546875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="17.85546875" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="17" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="28.85546875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="27.42578125" bestFit="1" customWidth="1" style="4" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="33.28515625" bestFit="1" customWidth="1" style="4" min="17" max="17"/>
+    <col width="41.7109375" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="48.85546875" bestFit="1" customWidth="1" style="4" min="19" max="19"/>
+    <col width="51.85546875" bestFit="1" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="30" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="40" customWidth="1" min="22" max="22"/>
+    <col width="79.85546875" bestFit="1" customWidth="1" style="4" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col hidden="1" width="40" customWidth="1" min="25" max="25"/>
+    <col width="79.85546875" bestFit="1" customWidth="1" style="4" min="26" max="26"/>
+    <col width="37" customWidth="1" min="27" max="27"/>
+    <col hidden="1" width="40" customWidth="1" min="28" max="28"/>
+    <col width="8.7109375" customWidth="1" min="29" max="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="4" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1" ht="15.75" customFormat="1" customHeight="1" s="4">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Host Name Onpremise</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>EC2 Name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Enviroment</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Number of CPUs</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>RAM (GB)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Operation System Type</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Operation System Name</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Instance Recommended</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>AWS Instance Deploy</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Total Cores</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>AWS RAM (GB)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>EBS Size (GB)</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>EBS Additional Size (GB)</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>AWS Region</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly Root EBS Cost</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr EBS Cost</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly Additional EBS Cost</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr Additional EBS Cost</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly  On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized License Only Cost</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized On-Demand EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly 1 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>Annualized 1 Yr NURI EC2 Cost, Excl. License Costs</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Monthly 3 Yr NURI  Standard Reserved Instances Total EC2 - RDS Cost</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI Total EC2 Cost</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>Annualized 3 Yr NURI EC2 Cost Excl. License Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>PAHWPAPSTS01</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>RHEL</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 8 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="3" t="s">
+      <c r="K2" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A2" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="6">
-        <v>4</v>
-      </c>
-      <c r="E2" s="6">
-        <v>16</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J2" s="6">
-        <v>2</v>
-      </c>
-      <c r="K2" s="6">
-        <v>16</v>
-      </c>
-      <c r="L2" s="6">
+      <c r="L2" s="6" t="n">
         <v>520</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="6">
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="n">
         <v>41.6</v>
       </c>
       <c r="P2" s="6">
-        <f t="shared" ref="P2:P3" si="0">PRODUCT(O2,12)</f>
-        <v>499.20000000000005</v>
-      </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6">
+        <f>PRODUCT(O2,12)</f>
+        <v/>
+      </c>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n">
         <v>104</v>
       </c>
       <c r="T2" s="6">
         <f>PRODUCT(S2,12)</f>
-        <v>1248</v>
-      </c>
-      <c r="U2" s="6">
+        <v/>
+      </c>
+      <c r="U2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="V2" s="6">
+      <c r="V2" s="6" t="n">
         <v>1244</v>
       </c>
-      <c r="W2" s="6">
+      <c r="W2" s="6" t="n">
         <v>73</v>
       </c>
       <c r="X2" s="6">
         <f>PRODUCT(W2,12)</f>
+        <v/>
+      </c>
+      <c r="Y2" s="6" t="n">
         <v>876</v>
       </c>
-      <c r="Y2" s="6">
-        <v>876</v>
-      </c>
-      <c r="Z2" s="6">
+      <c r="Z2" s="6" t="n">
         <v>57</v>
       </c>
       <c r="AA2" s="6">
         <f>PRODUCT(Z2,12)</f>
-        <v>684</v>
-      </c>
-      <c r="AB2" s="2">
+        <v/>
+      </c>
+      <c r="AB2" s="2" t="n">
         <v>683</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="6">
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>PAHWPAPSTE01</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" s="6">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>RHEL</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 8 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" s="6">
+      <c r="M3" s="6" t="n"/>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="n">
         <v>16.8</v>
       </c>
       <c r="P3" s="6">
-        <f t="shared" si="0"/>
-        <v>201.60000000000002</v>
-      </c>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6">
+        <f>PRODUCT(O3,12)</f>
+        <v/>
+      </c>
+      <c r="Q3" s="6" t="n"/>
+      <c r="R3" s="6" t="n"/>
+      <c r="S3" s="6" t="n">
         <v>104</v>
       </c>
       <c r="T3" s="6">
         <f>PRODUCT(S3,12)</f>
-        <v>1248</v>
-      </c>
-      <c r="U3" s="6">
+        <v/>
+      </c>
+      <c r="U3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="V3" s="6">
+      <c r="V3" s="6" t="n">
         <v>1244</v>
       </c>
-      <c r="W3" s="6">
+      <c r="W3" s="6" t="n">
         <v>73</v>
       </c>
       <c r="X3" s="6">
         <f>PRODUCT(W3,12)</f>
+        <v/>
+      </c>
+      <c r="Y3" s="6" t="n">
         <v>876</v>
       </c>
-      <c r="Y3" s="6">
-        <v>876</v>
-      </c>
-      <c r="Z3" s="6">
+      <c r="Z3" s="6" t="n">
         <v>57</v>
       </c>
       <c r="AA3" s="6">
-        <f t="shared" ref="AA3:AA17" si="1">PRODUCT(Z3,12)</f>
-        <v>684</v>
-      </c>
-      <c r="AB3" s="2">
+        <f>PRODUCT(Z3,12)</f>
+        <v/>
+      </c>
+      <c r="AB3" s="2" t="n">
         <v>683</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="30" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="6">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>PAHWPAPSRC03</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES23 
+USAEA1PWBWES24</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J4" s="6">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O4" s="6">
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="n">
         <v>9.6</v>
       </c>
       <c r="P4" s="6">
         <f>PRODUCT(O4,12)</f>
-        <v>115.19999999999999</v>
-      </c>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6">
+        <v/>
+      </c>
+      <c r="Q4" s="6" t="n"/>
+      <c r="R4" s="6" t="n"/>
+      <c r="S4" s="6" t="n">
         <v>149.65</v>
       </c>
       <c r="T4" s="6">
         <f>PRODUCT(S4,12)</f>
-        <v>1795.8000000000002</v>
-      </c>
-      <c r="U4" s="6">
+        <v/>
+      </c>
+      <c r="U4" s="6" t="n">
         <v>806</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="6" t="n">
         <v>990</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="6" t="n">
         <v>118.99</v>
       </c>
       <c r="X4" s="6">
         <f>PRODUCT(W4,12)</f>
-        <v>1427.8799999999999</v>
-      </c>
-      <c r="Y4" s="6">
+        <v/>
+      </c>
+      <c r="Y4" s="6" t="n">
         <v>622</v>
       </c>
-      <c r="Z4" s="6">
+      <c r="Z4" s="6" t="n">
         <v>102.93</v>
       </c>
       <c r="AA4" s="6">
-        <f t="shared" si="1"/>
-        <v>1235.1600000000001</v>
-      </c>
-      <c r="AB4" s="2">
+        <f>PRODUCT(Z4,12)</f>
+        <v/>
+      </c>
+      <c r="AB4" s="2" t="n">
         <v>569</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="30" customHeight="1">
-      <c r="A5" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="9">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPAPWFC01</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES25 
+USAEA1PWBWES26</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="9">
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" s="9">
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="n">
         <v>8</v>
       </c>
       <c r="P5" s="9">
-        <f t="shared" ref="P5:P18" si="2">PRODUCT(O5,12)</f>
-        <v>96</v>
-      </c>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9">
+        <f>PRODUCT(O5,12)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="9" t="n"/>
+      <c r="R5" s="9" t="n"/>
+      <c r="S5" s="9" t="n">
         <v>89.12</v>
       </c>
       <c r="T5" s="9">
-        <f t="shared" ref="T5:T18" si="3">PRODUCT(S5,12)</f>
-        <v>1069.44</v>
-      </c>
-      <c r="U5" s="9">
+        <f>PRODUCT(S5,12)</f>
+        <v/>
+      </c>
+      <c r="U5" s="9" t="n">
         <v>403</v>
       </c>
-      <c r="V5" s="9">
+      <c r="V5" s="9" t="n">
         <v>666</v>
       </c>
-      <c r="W5" s="9">
+      <c r="W5" s="9" t="n">
         <v>70.31</v>
       </c>
       <c r="X5" s="9">
-        <f t="shared" ref="X5:X17" si="4">PRODUCT(W5,12)</f>
-        <v>843.72</v>
-      </c>
-      <c r="Y5" s="9">
+        <f>PRODUCT(W5,12)</f>
+        <v/>
+      </c>
+      <c r="Y5" s="9" t="n">
         <v>441</v>
       </c>
-      <c r="Z5" s="9">
+      <c r="Z5" s="9" t="n">
         <v>58.77</v>
       </c>
       <c r="AA5" s="9">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB5" s="2">
+        <f>PRODUCT(Z5,12)</f>
+        <v/>
+      </c>
+      <c r="AB5" s="2" t="n">
         <v>302</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="6">
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>PAHWPWFINT01</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>USAEA1PFSWES09</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J6" s="6">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="N6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O6" s="6">
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="n">
         <v>8</v>
       </c>
       <c r="P6" s="6">
-        <f t="shared" si="2"/>
-        <v>96</v>
-      </c>
-      <c r="Q6" s="6">
+        <f>PRODUCT(O6,12)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="6" t="n">
         <v>24</v>
       </c>
       <c r="R6" s="6">
         <f>PRODUCT(Q6,12)</f>
-        <v>288</v>
-      </c>
-      <c r="S6" s="6">
+        <v/>
+      </c>
+      <c r="S6" s="6" t="n">
         <v>89.12</v>
       </c>
       <c r="T6" s="6">
-        <f t="shared" si="3"/>
-        <v>1069.44</v>
-      </c>
-      <c r="U6" s="6">
+        <f>PRODUCT(S6,12)</f>
+        <v/>
+      </c>
+      <c r="U6" s="6" t="n">
         <v>403</v>
       </c>
-      <c r="V6" s="6">
+      <c r="V6" s="6" t="n">
         <v>666</v>
       </c>
-      <c r="W6" s="6">
+      <c r="W6" s="6" t="n">
         <v>70.31</v>
       </c>
       <c r="X6" s="6">
-        <f t="shared" si="4"/>
-        <v>843.72</v>
-      </c>
-      <c r="Y6" s="6">
+        <f>PRODUCT(W6,12)</f>
+        <v/>
+      </c>
+      <c r="Y6" s="6" t="n">
         <v>441</v>
       </c>
-      <c r="Z6" s="6">
+      <c r="Z6" s="6" t="n">
         <v>58.77</v>
       </c>
       <c r="AA6" s="6">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB6" s="2">
+        <f>PRODUCT(Z6,12)</f>
+        <v/>
+      </c>
+      <c r="AB6" s="2" t="n">
         <v>302</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A7" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="9">
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPWSAPI01</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES35</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J7" s="9">
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="9" t="n">
         <v>120</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="N7" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O7" s="9">
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="n">
         <v>9.6</v>
       </c>
       <c r="P7" s="9">
-        <f t="shared" si="2"/>
-        <v>115.19999999999999</v>
-      </c>
-      <c r="Q7" s="9">
+        <f>PRODUCT(O7,12)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="9" t="n">
         <v>7.2</v>
       </c>
-      <c r="R7" s="9">
-        <v>86.4</v>
-      </c>
-      <c r="S7" s="9">
+      <c r="R7" s="9" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S7" s="9" t="n">
         <v>149.65</v>
       </c>
       <c r="T7" s="9">
-        <f t="shared" si="3"/>
-        <v>1795.8000000000002</v>
-      </c>
-      <c r="U7" s="9">
+        <f>PRODUCT(S7,12)</f>
+        <v/>
+      </c>
+      <c r="U7" s="9" t="n">
         <v>806</v>
       </c>
-      <c r="V7" s="9">
+      <c r="V7" s="9" t="n">
         <v>990</v>
       </c>
-      <c r="W7" s="9">
+      <c r="W7" s="9" t="n">
         <v>118.99</v>
       </c>
       <c r="X7" s="9">
-        <f t="shared" si="4"/>
-        <v>1427.8799999999999</v>
-      </c>
-      <c r="Y7" s="9">
+        <f>PRODUCT(W7,12)</f>
+        <v/>
+      </c>
+      <c r="Y7" s="9" t="n">
         <v>622</v>
       </c>
-      <c r="Z7" s="9">
+      <c r="Z7" s="9" t="n">
         <v>102.93</v>
       </c>
       <c r="AA7" s="9">
-        <f t="shared" si="1"/>
-        <v>1235.1600000000001</v>
-      </c>
-      <c r="AB7" s="2">
+        <f>PRODUCT(Z7,12)</f>
+        <v/>
+      </c>
+      <c r="AB7" s="2" t="n">
         <v>569</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="30" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="9">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPAPWSS03</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES27 
+USAEA1PWBWES28</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J8" s="9">
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O8" s="9">
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="n">
         <v>8</v>
       </c>
       <c r="P8" s="9">
-        <f t="shared" si="2"/>
-        <v>96</v>
-      </c>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9">
+        <f>PRODUCT(O8,12)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="9" t="n"/>
+      <c r="R8" s="9" t="n"/>
+      <c r="S8" s="9" t="n">
         <v>89.12</v>
       </c>
       <c r="T8" s="9">
-        <f t="shared" si="3"/>
-        <v>1069.44</v>
-      </c>
-      <c r="U8" s="9">
+        <f>PRODUCT(S8,12)</f>
+        <v/>
+      </c>
+      <c r="U8" s="9" t="n">
         <v>403</v>
       </c>
-      <c r="V8" s="9">
+      <c r="V8" s="9" t="n">
         <v>666</v>
       </c>
-      <c r="W8" s="9">
+      <c r="W8" s="9" t="n">
         <v>70.31</v>
       </c>
       <c r="X8" s="9">
-        <f t="shared" si="4"/>
-        <v>843.72</v>
-      </c>
-      <c r="Y8" s="9">
+        <f>PRODUCT(W8,12)</f>
+        <v/>
+      </c>
+      <c r="Y8" s="9" t="n">
         <v>441</v>
       </c>
-      <c r="Z8" s="9">
+      <c r="Z8" s="9" t="n">
         <v>58.77</v>
       </c>
       <c r="AA8" s="9">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB8" s="2">
+        <f>PRODUCT(Z8,12)</f>
+        <v/>
+      </c>
+      <c r="AB8" s="2" t="n">
         <v>302</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="9">
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPAPWEF02</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PAPWES34</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J9" s="9">
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="N9" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O9" s="9">
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="n">
         <v>8</v>
       </c>
       <c r="P9" s="9">
-        <f t="shared" si="2"/>
-        <v>96</v>
-      </c>
-      <c r="Q9" s="9">
+        <f>PRODUCT(O9,12)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="9" t="n">
         <v>7.2</v>
       </c>
-      <c r="R9" s="9">
-        <v>86.4</v>
-      </c>
-      <c r="S9" s="9">
+      <c r="R9" s="9" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S9" s="9" t="n">
         <v>89.12</v>
       </c>
       <c r="T9" s="9">
-        <f t="shared" si="3"/>
-        <v>1069.44</v>
-      </c>
-      <c r="U9" s="9">
+        <f>PRODUCT(S9,12)</f>
+        <v/>
+      </c>
+      <c r="U9" s="9" t="n">
         <v>403</v>
       </c>
-      <c r="V9" s="9">
+      <c r="V9" s="9" t="n">
         <v>666</v>
       </c>
-      <c r="W9" s="9">
+      <c r="W9" s="9" t="n">
         <v>70.31</v>
       </c>
       <c r="X9" s="9">
-        <f t="shared" si="4"/>
-        <v>843.72</v>
-      </c>
-      <c r="Y9" s="9">
+        <f>PRODUCT(W9,12)</f>
+        <v/>
+      </c>
+      <c r="Y9" s="9" t="n">
         <v>441</v>
       </c>
-      <c r="Z9" s="9">
+      <c r="Z9" s="9" t="n">
         <v>58.77</v>
       </c>
       <c r="AA9" s="9">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB9" s="2">
+        <f>PRODUCT(Z9,12)</f>
+        <v/>
+      </c>
+      <c r="AB9" s="2" t="n">
         <v>302</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="30.75" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="9">
+    <row r="10" ht="30.75" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPAPTUI03</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>USAEA1PWBWES21 
+USAEA1PWBWES22</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J10" s="9">
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit) [ASG app1 desplegado]</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O10" s="9">
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="n">
         <v>8</v>
       </c>
       <c r="P10" s="9">
-        <f t="shared" si="2"/>
-        <v>96</v>
-      </c>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9">
+        <f>PRODUCT(O10,12)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="9" t="n"/>
+      <c r="R10" s="9" t="n"/>
+      <c r="S10" s="9" t="n">
         <v>89.12</v>
       </c>
       <c r="T10" s="9">
-        <f t="shared" si="3"/>
-        <v>1069.44</v>
-      </c>
-      <c r="U10" s="9">
+        <f>PRODUCT(S10,12)</f>
+        <v/>
+      </c>
+      <c r="U10" s="9" t="n">
         <v>403</v>
       </c>
-      <c r="V10" s="9">
+      <c r="V10" s="9" t="n">
         <v>666</v>
       </c>
-      <c r="W10" s="9">
+      <c r="W10" s="9" t="n">
         <v>70.31</v>
       </c>
       <c r="X10" s="9">
-        <f t="shared" si="4"/>
-        <v>843.72</v>
-      </c>
-      <c r="Y10" s="9">
+        <f>PRODUCT(W10,12)</f>
+        <v/>
+      </c>
+      <c r="Y10" s="9" t="n">
         <v>441</v>
       </c>
-      <c r="Z10" s="9">
+      <c r="Z10" s="9" t="n">
         <v>58.77</v>
       </c>
       <c r="AA10" s="9">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB10" s="2">
+        <f>PRODUCT(Z10,12)</f>
+        <v/>
+      </c>
+      <c r="AB10" s="2" t="n">
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="30" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="9">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>PAHWPCHECS01</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PFSWES08</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" s="9">
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (64-bit)</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>r5a.large</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="9" t="n">
         <v>120</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="N11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O11" s="9">
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="n">
         <v>9.6</v>
       </c>
       <c r="P11" s="9">
-        <f t="shared" si="2"/>
-        <v>115.19999999999999</v>
-      </c>
-      <c r="Q11" s="9">
+        <f>PRODUCT(O11,12)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="9" t="n">
         <v>7.2</v>
       </c>
-      <c r="R11" s="9">
-        <v>86.4</v>
-      </c>
-      <c r="S11" s="9">
+      <c r="R11" s="9" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="S11" s="9" t="n">
         <v>149.65</v>
       </c>
       <c r="T11" s="9">
-        <f t="shared" si="3"/>
-        <v>1795.8000000000002</v>
-      </c>
-      <c r="U11" s="9">
+        <f>PRODUCT(S11,12)</f>
+        <v/>
+      </c>
+      <c r="U11" s="9" t="n">
         <v>806</v>
       </c>
-      <c r="V11" s="9">
+      <c r="V11" s="9" t="n">
         <v>990</v>
       </c>
-      <c r="W11" s="9">
+      <c r="W11" s="9" t="n">
         <v>118.99</v>
       </c>
       <c r="X11" s="9">
-        <f t="shared" si="4"/>
-        <v>1427.8799999999999</v>
-      </c>
-      <c r="Y11" s="9">
+        <f>PRODUCT(W11,12)</f>
+        <v/>
+      </c>
+      <c r="Y11" s="9" t="n">
         <v>622</v>
       </c>
-      <c r="Z11" s="9">
+      <c r="Z11" s="9" t="n">
         <v>102.93</v>
       </c>
       <c r="AA11" s="9">
-        <f t="shared" si="1"/>
-        <v>1235.1600000000001</v>
-      </c>
-      <c r="AB11" s="2">
+        <f>PRODUCT(Z11,12)</f>
+        <v/>
+      </c>
+      <c r="AB11" s="2" t="n">
         <v>569</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="9">
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>pahqpapapp02</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>USAEA1PAPWES33</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J12" s="9">
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Windows Server 2025 Standard</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>r7a.medium</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="9" t="n">
         <v>280</v>
       </c>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O12" s="9">
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="n">
         <v>22.4</v>
       </c>
       <c r="P12" s="9">
-        <f t="shared" si="2"/>
-        <v>268.79999999999995</v>
-      </c>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9">
+        <f>PRODUCT(O12,12)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="9" t="n"/>
+      <c r="R12" s="9" t="n"/>
+      <c r="S12" s="9" t="n">
         <v>89.12</v>
       </c>
       <c r="T12" s="9">
-        <f t="shared" si="3"/>
-        <v>1069.44</v>
-      </c>
-      <c r="U12" s="9">
+        <f>PRODUCT(S12,12)</f>
+        <v/>
+      </c>
+      <c r="U12" s="9" t="n">
         <v>402.96</v>
       </c>
-      <c r="V12" s="9">
+      <c r="V12" s="9" t="n">
         <v>666.46</v>
       </c>
-      <c r="W12" s="9">
+      <c r="W12" s="9" t="n">
         <v>70.31</v>
       </c>
       <c r="X12" s="9">
-        <f t="shared" si="4"/>
-        <v>843.72</v>
-      </c>
-      <c r="Y12" s="9">
+        <f>PRODUCT(W12,12)</f>
+        <v/>
+      </c>
+      <c r="Y12" s="9" t="n">
         <v>440.8</v>
       </c>
-      <c r="Z12" s="9">
+      <c r="Z12" s="9" t="n">
         <v>58.77</v>
       </c>
       <c r="AA12" s="9">
-        <f t="shared" si="1"/>
-        <v>705.24</v>
-      </c>
-      <c r="AB12" s="2">
+        <f>PRODUCT(Z12,12)</f>
+        <v/>
+      </c>
+      <c r="AB12" s="2" t="n">
         <v>302.31</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="9">
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>pahwpapbof01</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="J13" s="9">
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04.3 LTS TBD</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>c5a.large</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>c5a.large</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="9" t="n">
         <v>210</v>
       </c>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O13" s="9">
+      <c r="M13" s="9" t="n"/>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="n">
         <v>16.8</v>
       </c>
       <c r="P13" s="9">
-        <f t="shared" si="2"/>
-        <v>201.60000000000002</v>
-      </c>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9">
+        <f>PRODUCT(O13,12)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="9" t="n"/>
+      <c r="R13" s="9" t="n"/>
+      <c r="S13" s="9" t="n">
         <v>56.21</v>
       </c>
       <c r="T13" s="9">
-        <f t="shared" si="3"/>
+        <f>PRODUCT(S13,12)</f>
+        <v/>
+      </c>
+      <c r="U13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="9" t="n">
         <v>674.52</v>
       </c>
-      <c r="U13" s="9">
-        <v>0</v>
-      </c>
-      <c r="V13" s="9">
-        <v>674.52</v>
-      </c>
-      <c r="W13" s="9">
-        <v>35.770000000000003</v>
+      <c r="W13" s="9" t="n">
+        <v>35.77</v>
       </c>
       <c r="X13" s="9">
-        <f t="shared" si="4"/>
+        <f>PRODUCT(W13,12)</f>
+        <v/>
+      </c>
+      <c r="Y13" s="9" t="n">
         <v>429.24</v>
       </c>
-      <c r="Y13" s="9">
-        <v>429.24</v>
-      </c>
-      <c r="Z13" s="9">
+      <c r="Z13" s="9" t="n">
         <v>24.09</v>
       </c>
       <c r="AA13" s="9">
-        <f t="shared" si="1"/>
+        <f>PRODUCT(Z13,12)</f>
+        <v/>
+      </c>
+      <c r="AB13" s="2" t="n">
         <v>289.08</v>
       </c>
-      <c r="AB13" s="2">
-        <v>289.08</v>
-      </c>
     </row>
-    <row r="14" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="9">
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>RDS produccion (multiaz1)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="9" t="n">
         <v>128</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="J14" s="9">
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>SQL Server - Standard</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>SQL Server Standard Edition 15.x (Multi-AZ, license-included)</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>db.r6i.4xlarge</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>db.r6i.4xlarge</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="9" t="n">
         <v>128</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="9" t="n">
         <v>1700</v>
       </c>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O14" s="9">
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="n">
         <v>391</v>
       </c>
       <c r="P14" s="9">
-        <f t="shared" si="2"/>
-        <v>4692</v>
-      </c>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9">
-        <v>8876.7999999999993</v>
+        <f>PRODUCT(O14,12)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="9" t="n"/>
+      <c r="R14" s="9" t="n"/>
+      <c r="S14" s="9" t="n">
+        <v>8876.799999999999</v>
       </c>
       <c r="T14" s="9">
-        <f t="shared" si="3"/>
-        <v>106521.59999999999</v>
-      </c>
-      <c r="U14" s="9">
-        <v>54382.080000000002</v>
-      </c>
-      <c r="V14" s="9">
-        <v>52139.519999999997</v>
-      </c>
-      <c r="W14" s="9">
+        <f>PRODUCT(S14,12)</f>
+        <v/>
+      </c>
+      <c r="U14" s="9" t="n">
+        <v>54382.08</v>
+      </c>
+      <c r="V14" s="9" t="n">
+        <v>52139.52</v>
+      </c>
+      <c r="W14" s="9" t="n">
         <v>8388.58</v>
       </c>
       <c r="X14" s="9">
-        <f t="shared" si="4"/>
-        <v>100662.95999999999</v>
-      </c>
-      <c r="Y14" s="9"/>
+        <f>PRODUCT(W14,12)</f>
+        <v/>
+      </c>
+      <c r="Y14" s="9" t="n"/>
       <c r="Z14" s="9">
         <f>AA14/12</f>
-        <v>20878.25</v>
-      </c>
-      <c r="AA14" s="9">
+        <v/>
+      </c>
+      <c r="AA14" s="9" t="n">
         <v>250539</v>
       </c>
-      <c r="AB14" s="2" t="s">
-        <v>62</v>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="9">
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>RDS procesos (standalone1)</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="9" t="n">
         <v>64</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="9" t="s">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>SQL Server - Standard</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>SQL Server Standard Edition 15.x (Single-AZ, license-included)</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>db.r6i.2xlarge</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>db.r6i.2xlarge</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="9" t="n">
         <v>64</v>
       </c>
-      <c r="H15" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="J15" s="9">
-        <v>8</v>
-      </c>
-      <c r="K15" s="9">
-        <v>64</v>
-      </c>
-      <c r="L15" s="9">
+      <c r="L15" s="9" t="n">
         <v>2900</v>
       </c>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O15" s="9">
+      <c r="M15" s="9" t="n"/>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="n">
         <v>333.5</v>
       </c>
       <c r="P15" s="9">
-        <f t="shared" si="2"/>
-        <v>4002</v>
-      </c>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9">
-        <v>2219.1999999999998</v>
+        <f>PRODUCT(O15,12)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="9" t="n"/>
+      <c r="R15" s="9" t="n"/>
+      <c r="S15" s="9" t="n">
+        <v>2219.2</v>
       </c>
       <c r="T15" s="9">
-        <f t="shared" si="3"/>
-        <v>26630.399999999998</v>
-      </c>
-      <c r="U15" s="9">
+        <f>PRODUCT(S15,12)</f>
+        <v/>
+      </c>
+      <c r="U15" s="9" t="n">
         <v>13595.52</v>
       </c>
-      <c r="V15" s="9">
+      <c r="V15" s="9" t="n">
         <v>13034.88</v>
       </c>
-      <c r="W15" s="9">
+      <c r="W15" s="9" t="n">
         <v>2097.14</v>
       </c>
       <c r="X15" s="9">
-        <f t="shared" si="4"/>
-        <v>25165.68</v>
-      </c>
-      <c r="Y15" s="9"/>
+        <f>PRODUCT(W15,12)</f>
+        <v/>
+      </c>
+      <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="9">
         <f>AA15/12</f>
-        <v>5219.583333333333</v>
-      </c>
-      <c r="AA15" s="9">
+        <v/>
+      </c>
+      <c r="AA15" s="9" t="n">
         <v>62635</v>
       </c>
-      <c r="AB15" s="2" t="s">
-        <v>62</v>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A16" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6">
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>FSx Windows (intelisrcpa-prd)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Windows (FSx)</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>FSx Windows File Server Single-AZ SSD (64 MBps, backup 30d)</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>FSx SINGLE_AZ_1</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>FSx SINGLE_AZ_1</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O16" s="6"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="6"/>
-      <c r="S16" s="6">
-        <v>147.30000000000001</v>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+      <c r="Q16" s="6" t="n"/>
+      <c r="R16" s="6" t="n"/>
+      <c r="S16" s="6" t="n">
+        <v>147.3</v>
       </c>
       <c r="T16" s="6">
-        <f t="shared" si="3"/>
-        <v>1767.6000000000001</v>
-      </c>
-      <c r="U16" s="6">
+        <f>PRODUCT(S16,12)</f>
+        <v/>
+      </c>
+      <c r="U16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="V16" s="6">
+      <c r="V16" s="6" t="n">
         <v>1689.6</v>
       </c>
-      <c r="W16" s="6"/>
-      <c r="X16" s="6"/>
-      <c r="Y16" s="6"/>
-      <c r="Z16" s="6"/>
-      <c r="AA16" s="6"/>
-      <c r="AB16" s="2"/>
+      <c r="W16" s="6" t="n"/>
+      <c r="X16" s="6" t="n"/>
+      <c r="Y16" s="6" t="n"/>
+      <c r="Z16" s="6" t="n"/>
+      <c r="AA16" s="6" t="n"/>
+      <c r="AB16" s="2" t="n"/>
     </row>
-    <row r="17" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A17" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="6">
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>AMI Builder (temporal)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="J17" s="6">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft Windows Server 2025 (AMI Builder - temporal)</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>m5.large</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>m5.large</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O17" s="6">
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="n">
         <v>8</v>
       </c>
       <c r="P17" s="6">
-        <f t="shared" si="2"/>
-        <v>96</v>
-      </c>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="6">
+        <f>PRODUCT(O17,12)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="6" t="n"/>
+      <c r="R17" s="6" t="n"/>
+      <c r="S17" s="6" t="n">
         <v>137.24</v>
       </c>
       <c r="T17" s="6">
-        <f t="shared" si="3"/>
-        <v>1646.88</v>
-      </c>
-      <c r="U17" s="6">
+        <f>PRODUCT(S17,12)</f>
+        <v/>
+      </c>
+      <c r="U17" s="6" t="n">
         <v>805.92</v>
       </c>
-      <c r="V17" s="6">
+      <c r="V17" s="6" t="n">
         <v>840.96</v>
       </c>
-      <c r="W17" s="6">
+      <c r="W17" s="6" t="n">
         <v>110.96</v>
       </c>
       <c r="X17" s="6">
-        <f t="shared" si="4"/>
-        <v>1331.52</v>
-      </c>
-      <c r="Y17" s="6">
+        <f>PRODUCT(W17,12)</f>
+        <v/>
+      </c>
+      <c r="Y17" s="6" t="n">
         <v>525.6</v>
       </c>
-      <c r="Z17" s="6">
+      <c r="Z17" s="6" t="n">
         <v>97.09</v>
       </c>
       <c r="AA17" s="6">
-        <f t="shared" si="1"/>
-        <v>1165.08</v>
-      </c>
-      <c r="AB17" s="2">
+        <f>PRODUCT(Z17,12)</f>
+        <v/>
+      </c>
+      <c r="AB17" s="2" t="n">
         <v>359.16</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A18" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="6">
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>DMS replication</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="J18" s="6">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>DMS</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>DMS c5.2xlarge Single-AZ (engine 3.6.1)</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>dms.c5.2xlarge</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>dms.c5.2xlarge</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O18" s="6">
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="n">
         <v>5.75</v>
       </c>
       <c r="P18" s="6">
-        <f t="shared" si="2"/>
-        <v>69</v>
-      </c>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="6"/>
-      <c r="S18" s="6">
+        <f>PRODUCT(O18,12)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="6" t="n"/>
+      <c r="R18" s="6" t="n"/>
+      <c r="S18" s="6" t="n">
         <v>347.48</v>
       </c>
       <c r="T18" s="6">
-        <f t="shared" si="3"/>
+        <f>PRODUCT(S18,12)</f>
+        <v/>
+      </c>
+      <c r="U18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="6" t="n">
         <v>4169.76</v>
       </c>
-      <c r="U18" s="6">
-        <v>0</v>
-      </c>
-      <c r="V18" s="6">
-        <v>4169.76</v>
-      </c>
-      <c r="W18" s="6"/>
-      <c r="X18" s="6"/>
-      <c r="Y18" s="6"/>
-      <c r="Z18" s="6"/>
-      <c r="AA18" s="6"/>
-      <c r="AB18" s="2"/>
+      <c r="W18" s="6" t="n"/>
+      <c r="X18" s="6" t="n"/>
+      <c r="Y18" s="6" t="n"/>
+      <c r="Z18" s="6" t="n"/>
+      <c r="AA18" s="6" t="n"/>
+      <c r="AB18" s="2" t="n"/>
     </row>
-    <row r="20" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="21" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="22" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:28" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:28" ht="15.75" customHeight="1"/>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Application Load Balancer (eec-aws-us-eits-prod)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>ALB internal (4 TG/host-header)</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9" t="n"/>
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="9" t="n"/>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="n"/>
+      <c r="P19" s="9" t="n"/>
+      <c r="Q19" s="9" t="n"/>
+      <c r="R19" s="9" t="n"/>
+      <c r="S19" s="9" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="T19" s="9" t="n">
+        <v>477.36</v>
+      </c>
+      <c r="U19" s="9" t="n"/>
+      <c r="V19" s="9" t="n"/>
+      <c r="W19" s="9" t="n"/>
+      <c r="X19" s="9" t="n"/>
+      <c r="Y19" s="9" t="n"/>
+      <c r="Z19" s="9" t="n"/>
+      <c r="AA19" s="9" t="n"/>
+      <c r="AB19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>ASG Lifecycle (Lambda leave-domain)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Lambda py3.12 128MB + EventBridge + CW Logs</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="9" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="9" t="n"/>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="n"/>
+      <c r="P20" s="9" t="n"/>
+      <c r="Q20" s="9" t="n"/>
+      <c r="R20" s="9" t="n"/>
+      <c r="S20" s="9" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="T20" s="9" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="U20" s="9" t="n"/>
+      <c r="V20" s="9" t="n"/>
+      <c r="W20" s="9" t="n"/>
+      <c r="X20" s="9" t="n"/>
+      <c r="Y20" s="9" t="n"/>
+      <c r="Z20" s="9" t="n"/>
+      <c r="AA20" s="9" t="n"/>
+      <c r="AB20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>S3 (rds-backup + rds-ssis + backup-reports)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>3 buckets Standard</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="9" t="n"/>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="n"/>
+      <c r="P21" s="9" t="n"/>
+      <c r="Q21" s="9" t="n"/>
+      <c r="R21" s="9" t="n"/>
+      <c r="S21" s="9" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="T21" s="9" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="U21" s="9" t="n"/>
+      <c r="V21" s="9" t="n"/>
+      <c r="W21" s="9" t="n"/>
+      <c r="X21" s="9" t="n"/>
+      <c r="Y21" s="9" t="n"/>
+      <c r="Z21" s="9" t="n"/>
+      <c r="AA21" s="9" t="n"/>
+      <c r="AB21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Secrets Manager (AD/DMS credentials)</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>5 secrets</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="n"/>
+      <c r="P22" s="9" t="n"/>
+      <c r="Q22" s="9" t="n"/>
+      <c r="R22" s="9" t="n"/>
+      <c r="S22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="T22" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="U22" s="9" t="n"/>
+      <c r="V22" s="9" t="n"/>
+      <c r="W22" s="9" t="n"/>
+      <c r="X22" s="9" t="n"/>
+      <c r="Y22" s="9" t="n"/>
+      <c r="Z22" s="9" t="n"/>
+      <c r="AA22" s="9" t="n"/>
+      <c r="AB22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>CloudWatch (alarmas ALB/ASG + metricas)</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>8 alarmas</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>US East (N. Virginia)</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="n"/>
+      <c r="P23" s="9" t="n"/>
+      <c r="Q23" s="9" t="n"/>
+      <c r="R23" s="9" t="n"/>
+      <c r="S23" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T23" s="9" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="U23" s="9" t="n"/>
+      <c r="V23" s="9" t="n"/>
+      <c r="W23" s="9" t="n"/>
+      <c r="X23" s="9" t="n"/>
+      <c r="Y23" s="9" t="n"/>
+      <c r="Z23" s="9" t="n"/>
+      <c r="AA23" s="9" t="n"/>
+      <c r="AB23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -5495,6 +5903,6 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>